<commit_message>
Add supplier-credit cash flow sheet and payment-term parameters
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W6G8eVwxeF9fr6fyaH3NLi
</commit_message>
<xml_diff>
--- a/central-loja/planilha_gestao_loja.xlsx
+++ b/central-loja/planilha_gestao_loja.xlsx
@@ -13,8 +13,9 @@
     <sheet name="Custos_SKU" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Ads" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Estoque" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Resultado" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Simulador" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Fluxo_Caixa" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Resultado" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Simulador" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="176">
   <si>
     <t xml:space="preserve">Central de Gestão da Loja – Planilha base (v0.4)</t>
   </si>
@@ -58,6 +59,9 @@
     <t xml:space="preserve">Estoque – cobertura em dias e ponto de reposição por SKU (você não usa ERP; esta é a fonte única de estoque).</t>
   </si>
   <si>
+    <t xml:space="preserve">Fluxo_Caixa – boletos de compra (30 dias) x entradas do ML mês a mês: mostra se o lucro virou caixa.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resultado – lucro líquido mensal e acumulado contra a meta.</t>
   </si>
   <si>
@@ -184,6 +188,24 @@
     <t xml:space="preserve">HIPÓTESE – ajustar conforme variação real da demanda.</t>
   </si>
   <si>
+    <t xml:space="preserve">Prazo de pagamento ao fornecedor (dias)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Informado: compra a prazo, boleto de 30 dias.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limite de crédito com o fornecedor (R$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A PREENCHER: quanto o fornecedor permite comprar a prazo. Zero = desconhecido.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prazo de liberação dos valores pelo ML (dias)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A PREENCHER com o prazo real do seu Painel (não presumido).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Custos e margem por SKU / canal</t>
   </si>
   <si>
@@ -361,30 +383,78 @@
     <t xml:space="preserve">Capital total necessário para repor 30 dias:</t>
   </si>
   <si>
-    <t xml:space="preserve">Capital disponível (Parametros):</t>
+    <t xml:space="preserve">Capital próprio + crédito do fornecedor (Parametros):</t>
   </si>
   <si>
     <t xml:space="preserve">Saldo (negativo = capital insuficiente):</t>
   </si>
   <si>
+    <t xml:space="preserve">Fluxo de caixa: boletos de compra x entradas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compras a prazo (boleto em 30 dias): a compra do mês M vence no mês M+1. O lucro só vira caixa se as entradas do ML cobrirem os boletos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo inicial de caixa (R$):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mês 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mês 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mês 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mês 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(+) Entradas líquidas liberadas pelo ML (já sem tarifas, frete e Ads)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(-) Boletos vencendo no mês</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(-) Impostos pagos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(-) Custos fixos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(-) Embalagem paga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(=) Caixa do mês</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caixa acumulado (inclui saldo inicial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compras do mês (boletos gerados, vencem no mês seguinte)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dívida de fornecedor em aberto no fim do mês</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crédito de fornecedor ainda disponível</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mês 1: preencha em 'Boletos vencendo' os boletos de compras de antes do início do controle. Impostos e embalagem: valores efetivamente pagos no mês.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se 'Limite de crédito' em Parametros estiver zerado, a linha de crédito disponível não tem significado.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lucro líquido mensal x meta</t>
   </si>
   <si>
     <t xml:space="preserve">Preencha as linhas azuis a cada mês com os valores reais do Painel e da contabilidade. Imposto e custos fixos vêm dos Parametros.</t>
   </si>
   <si>
-    <t xml:space="preserve">Item</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mês 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mês 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mês 3</t>
-  </si>
-  <si>
     <t xml:space="preserve">Total</t>
   </si>
   <si>
@@ -419,9 +489,6 @@
   </si>
   <si>
     <t xml:space="preserve">Margem de contribuição (% do faturamento)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(-) Custos fixos</t>
   </si>
   <si>
     <t xml:space="preserve">(=) LUCRO LÍQUIDO DO MÊS</t>
@@ -1051,7 +1118,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -1124,15 +1191,15 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3"/>
+      <c r="A15" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
-        <v>12</v>
-      </c>
+      <c r="A16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1157,16 +1224,21 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3"/>
+      <c r="A22" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>18</v>
-      </c>
+      <c r="A23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="2" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1185,7 +1257,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -1195,196 +1267,229 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>0.04</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" s="7" t="n">
         <v>0.15</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>0.08</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B7" s="9" t="n">
         <v>5000</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B8" s="10" t="n">
         <v>3</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B9" s="9" t="n">
         <v>300</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B10" s="11" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B11" s="12" t="n">
         <f aca="false">B9+B10</f>
         <v>300</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">100/35</f>
         <v>2.85714285714286</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B13" s="13" t="n">
         <v>0</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B14" s="9" t="n">
         <v>105</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B15" s="10" t="n">
         <v>35</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B16" s="9" t="n">
         <v>500</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B17" s="10" t="n">
         <v>25</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B18" s="9" t="n">
         <v>50</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B19" s="14" t="n">
         <v>10</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1425,91 +1530,91 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="P5" s="5" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="Q5" s="5" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="R5" s="5" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="S5" s="5" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="T5" s="5" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>100</v>
@@ -1538,7 +1643,7 @@
         <v>3</v>
       </c>
       <c r="M6" s="16" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="N6" s="12" t="n">
         <f aca="false">IF($E6="","",E6*Parametros!$B$4)</f>
@@ -3168,70 +3273,70 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="D6" s="14" t="n">
         <v>10000</v>
@@ -4381,7 +4486,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="D36" s="20" t="n">
         <f aca="false">SUM(D6:D35)</f>
@@ -4468,55 +4573,55 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C6" s="14" t="n">
         <v>30</v>
@@ -5363,7 +5468,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="26" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="I37" s="21" t="n">
         <f aca="false">SUM(I6:I35)</f>
@@ -5372,16 +5477,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="26" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="I38" s="12" t="n">
-        <f aca="false">Parametros!$B$16</f>
+        <f aca="false">Parametros!$B$16+Parametros!$B$21</f>
         <v>500</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="26" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="I39" s="21" t="n">
         <f aca="false">I38-I37</f>
@@ -5412,353 +5517,219 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>114</v>
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="27" t="n">
-        <f aca="false">SUM(B5:D5)</f>
-        <v>0</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
+      <c r="C6" s="12" t="n">
+        <f aca="false">B12</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="12" t="n">
+        <f aca="false">C12</f>
+        <v>0</v>
+      </c>
       <c r="E6" s="12" t="n">
-        <f aca="false">SUM(B6:D6)</f>
+        <f aca="false">D12</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
       <c r="D7" s="11"/>
-      <c r="E7" s="12" t="n">
-        <f aca="false">SUM(B7:D7)</f>
-        <v>0</v>
-      </c>
+      <c r="E7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
+        <v>131</v>
+      </c>
+      <c r="B8" s="12" t="n">
+        <f aca="false">Parametros!$B$11</f>
+        <v>300</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <f aca="false">Parametros!$B$11</f>
+        <v>300</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <f aca="false">Parametros!$B$11</f>
+        <v>300</v>
+      </c>
       <c r="E8" s="12" t="n">
-        <f aca="false">SUM(B8:D8)</f>
-        <v>0</v>
+        <f aca="false">Parametros!$B$11</f>
+        <v>300</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
       <c r="D9" s="11"/>
-      <c r="E9" s="12" t="n">
-        <f aca="false">SUM(B9:D9)</f>
-        <v>0</v>
-      </c>
+      <c r="E9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="12" t="n">
-        <f aca="false">SUM(B10:D10)</f>
-        <v>0</v>
+      <c r="A10" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="B10" s="21" t="n">
+        <f aca="false">B5-SUM(B6:B9)</f>
+        <v>-300</v>
+      </c>
+      <c r="C10" s="21" t="n">
+        <f aca="false">C5-SUM(C6:C9)</f>
+        <v>-300</v>
+      </c>
+      <c r="D10" s="21" t="n">
+        <f aca="false">D5-SUM(D6:D9)</f>
+        <v>-300</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <f aca="false">E5-SUM(E6:E9)</f>
+        <v>-300</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="12" t="n">
-        <f aca="false">SUM(B11:D11)</f>
-        <v>0</v>
+      <c r="A11" s="19" t="s">
+        <v>134</v>
+      </c>
+      <c r="B11" s="21" t="n">
+        <f aca="false">$B$3+B10</f>
+        <v>-300</v>
+      </c>
+      <c r="C11" s="21" t="n">
+        <f aca="false">B11+C10</f>
+        <v>-600</v>
+      </c>
+      <c r="D11" s="21" t="n">
+        <f aca="false">C11+D10</f>
+        <v>-900</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <f aca="false">D11+E10</f>
+        <v>-1200</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="B12" s="12" t="n">
-        <f aca="false">B6*Parametros!$B$4</f>
-        <v>0</v>
-      </c>
-      <c r="C12" s="12" t="n">
-        <f aca="false">C6*Parametros!$B$4</f>
-        <v>0</v>
-      </c>
-      <c r="D12" s="12" t="n">
-        <f aca="false">D6*Parametros!$B$4</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="12" t="n">
-        <f aca="false">SUM(B12:D12)</f>
-        <v>0</v>
-      </c>
+        <v>135</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
+        <v>136</v>
+      </c>
+      <c r="B13" s="12" t="n">
+        <f aca="false">B12</f>
+        <v>0</v>
+      </c>
+      <c r="C13" s="12" t="n">
+        <f aca="false">C12</f>
+        <v>0</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <f aca="false">D12</f>
+        <v>0</v>
+      </c>
       <c r="E13" s="12" t="n">
-        <f aca="false">SUM(B13:D13)</f>
+        <f aca="false">E12</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
-        <v>129</v>
-      </c>
-      <c r="B14" s="21" t="n">
-        <f aca="false">B6-SUM(B7:B13)</f>
-        <v>0</v>
-      </c>
-      <c r="C14" s="21" t="n">
-        <f aca="false">C6-SUM(C7:C13)</f>
-        <v>0</v>
-      </c>
-      <c r="D14" s="21" t="n">
-        <f aca="false">D6-SUM(D7:D13)</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="21" t="n">
-        <f aca="false">SUM(B14:D14)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="B15" s="17" t="str">
-        <f aca="false">IF(B6&gt;0,B14/B6,"")</f>
-        <v/>
-      </c>
-      <c r="C15" s="17" t="str">
-        <f aca="false">IF(C6&gt;0,C14/C6,"")</f>
-        <v/>
-      </c>
-      <c r="D15" s="17" t="str">
-        <f aca="false">IF(D6&gt;0,D14/D6,"")</f>
-        <v/>
-      </c>
-      <c r="E15" s="17" t="str">
-        <f aca="false">IF(E6&gt;0,E14/E6,"")</f>
-        <v/>
+      <c r="A14" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B14" s="12" t="n">
+        <f aca="false">MAX(0,Parametros!$B$21-B13)</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="12" t="n">
+        <f aca="false">MAX(0,Parametros!$B$21-C13)</f>
+        <v>0</v>
+      </c>
+      <c r="D14" s="12" t="n">
+        <f aca="false">MAX(0,Parametros!$B$21-D13)</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <f aca="false">MAX(0,Parametros!$B$21-E13)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="B16" s="12" t="n">
-        <f aca="false">Parametros!$B$11</f>
-        <v>300</v>
-      </c>
-      <c r="C16" s="12" t="n">
-        <f aca="false">Parametros!$B$11</f>
-        <v>300</v>
-      </c>
-      <c r="D16" s="12" t="n">
-        <f aca="false">Parametros!$B$11</f>
-        <v>300</v>
-      </c>
-      <c r="E16" s="12" t="n">
-        <f aca="false">SUM(B16:D16)</f>
-        <v>900</v>
+      <c r="A16" s="15" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="B17" s="21" t="n">
-        <f aca="false">B14-B16</f>
-        <v>-300</v>
-      </c>
-      <c r="C17" s="21" t="n">
-        <f aca="false">C14-C16</f>
-        <v>-300</v>
-      </c>
-      <c r="D17" s="21" t="n">
-        <f aca="false">D14-D16</f>
-        <v>-300</v>
-      </c>
-      <c r="E17" s="21" t="n">
-        <f aca="false">SUM(B17:D17)</f>
-        <v>-900</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="B18" s="12" t="n">
-        <f aca="false">SUM($B17:B17)</f>
-        <v>-300</v>
-      </c>
-      <c r="C18" s="12" t="n">
-        <f aca="false">SUM($B17:C17)</f>
-        <v>-600</v>
-      </c>
-      <c r="D18" s="12" t="n">
-        <f aca="false">SUM($B17:D17)</f>
-        <v>-900</v>
-      </c>
-      <c r="E18" s="12" t="n">
-        <f aca="false">E17</f>
-        <v>-900</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="B19" s="12" t="n">
-        <f aca="false">Parametros!$B$7-B18</f>
-        <v>5300</v>
-      </c>
-      <c r="C19" s="12" t="n">
-        <f aca="false">Parametros!$B$7-C18</f>
-        <v>5600</v>
-      </c>
-      <c r="D19" s="12" t="n">
-        <f aca="false">Parametros!$B$7-D18</f>
-        <v>5900</v>
-      </c>
-      <c r="E19" s="12" t="n">
-        <f aca="false">Parametros!$B$7-E17</f>
-        <v>5900</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="B20" s="17" t="n">
-        <f aca="false">IF(Parametros!$B$7&gt;0,B18/Parametros!$B$7,"")</f>
-        <v>-0.06</v>
-      </c>
-      <c r="C20" s="17" t="n">
-        <f aca="false">IF(Parametros!$B$7&gt;0,C18/Parametros!$B$7,"")</f>
-        <v>-0.12</v>
-      </c>
-      <c r="D20" s="17" t="n">
-        <f aca="false">IF(Parametros!$B$7&gt;0,D18/Parametros!$B$7,"")</f>
-        <v>-0.18</v>
-      </c>
-      <c r="E20" s="17" t="n">
-        <f aca="false">IF(Parametros!$B$7&gt;0,E17/Parametros!$B$7,"")</f>
-        <v>-0.18</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="B21" s="12" t="str">
-        <f aca="false">IF(B5&gt;0,B6/B5,"")</f>
-        <v/>
-      </c>
-      <c r="C21" s="12" t="str">
-        <f aca="false">IF(C5&gt;0,C6/C5,"")</f>
-        <v/>
-      </c>
-      <c r="D21" s="12" t="str">
-        <f aca="false">IF(D5&gt;0,D6/D5,"")</f>
-        <v/>
-      </c>
-      <c r="E21" s="12" t="str">
-        <f aca="false">IF(E5&gt;0,E6/E5,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="B22" s="17" t="str">
-        <f aca="false">IF(B6&gt;0,B13/B6,"")</f>
-        <v/>
-      </c>
-      <c r="C22" s="17" t="str">
-        <f aca="false">IF(C6&gt;0,C13/C6,"")</f>
-        <v/>
-      </c>
-      <c r="D22" s="17" t="str">
-        <f aca="false">IF(D6&gt;0,D13/D6,"")</f>
-        <v/>
-      </c>
-      <c r="E22" s="17" t="str">
-        <f aca="false">IF(E6&gt;0,E13/E6,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="s">
-        <v>138</v>
+      <c r="A17" s="15" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B17:E17">
+  <conditionalFormatting sqref="B10:E11">
     <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>0</formula>
     </cfRule>
@@ -5778,6 +5749,372 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:E24"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="15" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="27" t="n">
+        <f aca="false">SUM(B5:D5)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="12" t="n">
+        <f aca="false">SUM(B6:D6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="12" t="n">
+        <f aca="false">SUM(B7:D7)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="12" t="n">
+        <f aca="false">SUM(B8:D8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="12" t="n">
+        <f aca="false">SUM(B9:D9)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="12" t="n">
+        <f aca="false">SUM(B10:D10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="12" t="n">
+        <f aca="false">SUM(B11:D11)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="B12" s="12" t="n">
+        <f aca="false">B6*Parametros!$B$4</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="12" t="n">
+        <f aca="false">C6*Parametros!$B$4</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="12" t="n">
+        <f aca="false">D6*Parametros!$B$4</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <f aca="false">SUM(B12:D12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="12" t="n">
+        <f aca="false">SUM(B13:D13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="B14" s="21" t="n">
+        <f aca="false">B6-SUM(B7:B13)</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="21" t="n">
+        <f aca="false">C6-SUM(C7:C13)</f>
+        <v>0</v>
+      </c>
+      <c r="D14" s="21" t="n">
+        <f aca="false">D6-SUM(D7:D13)</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="21" t="n">
+        <f aca="false">SUM(B14:D14)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="B15" s="17" t="str">
+        <f aca="false">IF(B6&gt;0,B14/B6,"")</f>
+        <v/>
+      </c>
+      <c r="C15" s="17" t="str">
+        <f aca="false">IF(C6&gt;0,C14/C6,"")</f>
+        <v/>
+      </c>
+      <c r="D15" s="17" t="str">
+        <f aca="false">IF(D6&gt;0,D14/D6,"")</f>
+        <v/>
+      </c>
+      <c r="E15" s="17" t="str">
+        <f aca="false">IF(E6&gt;0,E14/E6,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="B16" s="12" t="n">
+        <f aca="false">Parametros!$B$11</f>
+        <v>300</v>
+      </c>
+      <c r="C16" s="12" t="n">
+        <f aca="false">Parametros!$B$11</f>
+        <v>300</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <f aca="false">Parametros!$B$11</f>
+        <v>300</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <f aca="false">SUM(B16:D16)</f>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="B17" s="21" t="n">
+        <f aca="false">B14-B16</f>
+        <v>-300</v>
+      </c>
+      <c r="C17" s="21" t="n">
+        <f aca="false">C14-C16</f>
+        <v>-300</v>
+      </c>
+      <c r="D17" s="21" t="n">
+        <f aca="false">D14-D16</f>
+        <v>-300</v>
+      </c>
+      <c r="E17" s="21" t="n">
+        <f aca="false">SUM(B17:D17)</f>
+        <v>-900</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B18" s="12" t="n">
+        <f aca="false">SUM($B17:B17)</f>
+        <v>-300</v>
+      </c>
+      <c r="C18" s="12" t="n">
+        <f aca="false">SUM($B17:C17)</f>
+        <v>-600</v>
+      </c>
+      <c r="D18" s="12" t="n">
+        <f aca="false">SUM($B17:D17)</f>
+        <v>-900</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <f aca="false">E17</f>
+        <v>-900</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="B19" s="12" t="n">
+        <f aca="false">Parametros!$B$7-B18</f>
+        <v>5300</v>
+      </c>
+      <c r="C19" s="12" t="n">
+        <f aca="false">Parametros!$B$7-C18</f>
+        <v>5600</v>
+      </c>
+      <c r="D19" s="12" t="n">
+        <f aca="false">Parametros!$B$7-D18</f>
+        <v>5900</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <f aca="false">Parametros!$B$7-E17</f>
+        <v>5900</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="B20" s="17" t="n">
+        <f aca="false">IF(Parametros!$B$7&gt;0,B18/Parametros!$B$7,"")</f>
+        <v>-0.06</v>
+      </c>
+      <c r="C20" s="17" t="n">
+        <f aca="false">IF(Parametros!$B$7&gt;0,C18/Parametros!$B$7,"")</f>
+        <v>-0.12</v>
+      </c>
+      <c r="D20" s="17" t="n">
+        <f aca="false">IF(Parametros!$B$7&gt;0,D18/Parametros!$B$7,"")</f>
+        <v>-0.18</v>
+      </c>
+      <c r="E20" s="17" t="n">
+        <f aca="false">IF(Parametros!$B$7&gt;0,E17/Parametros!$B$7,"")</f>
+        <v>-0.18</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="B21" s="12" t="str">
+        <f aca="false">IF(B5&gt;0,B6/B5,"")</f>
+        <v/>
+      </c>
+      <c r="C21" s="12" t="str">
+        <f aca="false">IF(C5&gt;0,C6/C5,"")</f>
+        <v/>
+      </c>
+      <c r="D21" s="12" t="str">
+        <f aca="false">IF(D5&gt;0,D6/D5,"")</f>
+        <v/>
+      </c>
+      <c r="E21" s="12" t="str">
+        <f aca="false">IF(E5&gt;0,E6/E5,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="B22" s="17" t="str">
+        <f aca="false">IF(B6&gt;0,B13/B6,"")</f>
+        <v/>
+      </c>
+      <c r="C22" s="17" t="str">
+        <f aca="false">IF(C6&gt;0,C13/C6,"")</f>
+        <v/>
+      </c>
+      <c r="D22" s="17" t="str">
+        <f aca="false">IF(D6&gt;0,D13/D6,"")</f>
+        <v/>
+      </c>
+      <c r="E22" s="17" t="str">
+        <f aca="false">IF(E6&gt;0,E13/E6,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="15" t="s">
+        <v>160</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B17:E17">
+    <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:G15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -5790,17 +6127,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="28" t="s">
-        <v>141</v>
+        <v>163</v>
       </c>
       <c r="B4" s="12" t="n">
         <f aca="false">Parametros!$B$7/Parametros!$B$8</f>
@@ -5809,7 +6146,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
-        <v>142</v>
+        <v>164</v>
       </c>
       <c r="B5" s="12" t="n">
         <f aca="false">Parametros!$B$11</f>
@@ -5818,7 +6155,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="28" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="B6" s="21" t="n">
         <f aca="false">B4+B5</f>
@@ -5827,7 +6164,7 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="29" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="B7" s="12" t="n">
         <f aca="false">2*Parametros!$B$7/(Parametros!$B$8+1)</f>
@@ -5836,7 +6173,7 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="29" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="B8" s="21" t="n">
         <f aca="false">B7+B5</f>
@@ -5845,25 +6182,25 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>147</v>
+        <v>169</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>149</v>
+        <v>171</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>150</v>
+        <v>172</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>151</v>
+        <v>173</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>152</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5955,7 +6292,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>153</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add fixed-fee parameters (unconfirmed estimate) to cost sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W6G8eVwxeF9fr6fyaH3NLi
</commit_message>
<xml_diff>
--- a/central-loja/planilha_gestao_loja.xlsx
+++ b/central-loja/planilha_gestao_loja.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="180">
   <si>
     <t xml:space="preserve">Central de Gestão da Loja – Planilha base (v0.4)</t>
   </si>
@@ -71,7 +71,7 @@
     <t xml:space="preserve">REGRAS DE DADOS</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Comissão, tarifa fixa e frete NÃO foram presumidos: copie-os do Painel (relatório de vendas / detalhe da tarifa) para cada anúncio.</t>
+    <t xml:space="preserve">1. Comissão e frete NÃO foram presumidos: copie-os do Painel para cada anúncio. A tarifa fixa (coluna H) usa uma HIPÓTESE de fontes de terceiros (Parametros B23:B24) e deve ser conferida no simulador oficial do Mercado Livre; sobrescreva a fórmula com o valor real.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Preencha a coluna 'Origem do dado' (Real, Estimativa ou Hipótese). Só 'Real' sustenta decisões; as demais exigem validação.</t>
@@ -204,6 +204,18 @@
   </si>
   <si>
     <t xml:space="preserve">A PREENCHER com o prazo real do seu Painel (não presumido).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarifa fixa por unidade (R$) para preço abaixo do limite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HIPÓTESE NÃO CONFIRMADA: blogs de terceiros citam R$ 6,25–6,75 (ponto médio) e, desde 02/03/2026, valor variável por peso/dimensão (~R$ 6–7 típico). Confirmar no simulador oficial do ML.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preço abaixo do qual a tarifa fixa se aplica (R$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HIPÓTESE NÃO CONFIRMADA: fontes de terceiros citam R$ 79. Conferir no Painel.</t>
   </si>
   <si>
     <t xml:space="preserve">Custos e margem por SKU / canal</t>
@@ -1203,7 +1215,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
         <v>14</v>
       </c>
@@ -1257,7 +1269,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -1490,6 +1502,28 @@
       </c>
       <c r="C22" s="8" t="s">
         <v>58</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" s="11" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="11" t="n">
+        <v>79</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1530,91 +1564,91 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="P5" s="5" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="Q5" s="5" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="R5" s="5" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="S5" s="5" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="T5" s="5" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>100</v>
@@ -1626,6 +1660,7 @@
         <v>0.14</v>
       </c>
       <c r="H6" s="11" t="n">
+        <f aca="false">IF(E6="","",IF(E6&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
         <v>0</v>
       </c>
       <c r="I6" s="11" t="n">
@@ -1643,7 +1678,7 @@
         <v>3</v>
       </c>
       <c r="M6" s="16" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="N6" s="12" t="n">
         <f aca="false">IF($E6="","",E6*Parametros!$B$4)</f>
@@ -1686,7 +1721,10 @@
       <c r="E7" s="11"/>
       <c r="F7" s="11"/>
       <c r="G7" s="13"/>
-      <c r="H7" s="11"/>
+      <c r="H7" s="11" t="str">
+        <f aca="false">IF(E7="","",IF(E7&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I7" s="11"/>
       <c r="J7" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -1739,7 +1777,10 @@
       <c r="E8" s="11"/>
       <c r="F8" s="11"/>
       <c r="G8" s="13"/>
-      <c r="H8" s="11"/>
+      <c r="H8" s="11" t="str">
+        <f aca="false">IF(E8="","",IF(E8&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I8" s="11"/>
       <c r="J8" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -1792,7 +1833,10 @@
       <c r="E9" s="11"/>
       <c r="F9" s="11"/>
       <c r="G9" s="13"/>
-      <c r="H9" s="11"/>
+      <c r="H9" s="11" t="str">
+        <f aca="false">IF(E9="","",IF(E9&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I9" s="11"/>
       <c r="J9" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -1845,7 +1889,10 @@
       <c r="E10" s="11"/>
       <c r="F10" s="11"/>
       <c r="G10" s="13"/>
-      <c r="H10" s="11"/>
+      <c r="H10" s="11" t="str">
+        <f aca="false">IF(E10="","",IF(E10&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I10" s="11"/>
       <c r="J10" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -1898,7 +1945,10 @@
       <c r="E11" s="11"/>
       <c r="F11" s="11"/>
       <c r="G11" s="13"/>
-      <c r="H11" s="11"/>
+      <c r="H11" s="11" t="str">
+        <f aca="false">IF(E11="","",IF(E11&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I11" s="11"/>
       <c r="J11" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -1951,7 +2001,10 @@
       <c r="E12" s="11"/>
       <c r="F12" s="11"/>
       <c r="G12" s="13"/>
-      <c r="H12" s="11"/>
+      <c r="H12" s="11" t="str">
+        <f aca="false">IF(E12="","",IF(E12&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I12" s="11"/>
       <c r="J12" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2004,7 +2057,10 @@
       <c r="E13" s="11"/>
       <c r="F13" s="11"/>
       <c r="G13" s="13"/>
-      <c r="H13" s="11"/>
+      <c r="H13" s="11" t="str">
+        <f aca="false">IF(E13="","",IF(E13&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I13" s="11"/>
       <c r="J13" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2057,7 +2113,10 @@
       <c r="E14" s="11"/>
       <c r="F14" s="11"/>
       <c r="G14" s="13"/>
-      <c r="H14" s="11"/>
+      <c r="H14" s="11" t="str">
+        <f aca="false">IF(E14="","",IF(E14&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I14" s="11"/>
       <c r="J14" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2110,7 +2169,10 @@
       <c r="E15" s="11"/>
       <c r="F15" s="11"/>
       <c r="G15" s="13"/>
-      <c r="H15" s="11"/>
+      <c r="H15" s="11" t="str">
+        <f aca="false">IF(E15="","",IF(E15&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I15" s="11"/>
       <c r="J15" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2163,7 +2225,10 @@
       <c r="E16" s="11"/>
       <c r="F16" s="11"/>
       <c r="G16" s="13"/>
-      <c r="H16" s="11"/>
+      <c r="H16" s="11" t="str">
+        <f aca="false">IF(E16="","",IF(E16&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I16" s="11"/>
       <c r="J16" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2216,7 +2281,10 @@
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
       <c r="G17" s="13"/>
-      <c r="H17" s="11"/>
+      <c r="H17" s="11" t="str">
+        <f aca="false">IF(E17="","",IF(E17&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I17" s="11"/>
       <c r="J17" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2269,7 +2337,10 @@
       <c r="E18" s="11"/>
       <c r="F18" s="11"/>
       <c r="G18" s="13"/>
-      <c r="H18" s="11"/>
+      <c r="H18" s="11" t="str">
+        <f aca="false">IF(E18="","",IF(E18&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I18" s="11"/>
       <c r="J18" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2322,7 +2393,10 @@
       <c r="E19" s="11"/>
       <c r="F19" s="11"/>
       <c r="G19" s="13"/>
-      <c r="H19" s="11"/>
+      <c r="H19" s="11" t="str">
+        <f aca="false">IF(E19="","",IF(E19&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I19" s="11"/>
       <c r="J19" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2375,7 +2449,10 @@
       <c r="E20" s="11"/>
       <c r="F20" s="11"/>
       <c r="G20" s="13"/>
-      <c r="H20" s="11"/>
+      <c r="H20" s="11" t="str">
+        <f aca="false">IF(E20="","",IF(E20&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I20" s="11"/>
       <c r="J20" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2428,7 +2505,10 @@
       <c r="E21" s="11"/>
       <c r="F21" s="11"/>
       <c r="G21" s="13"/>
-      <c r="H21" s="11"/>
+      <c r="H21" s="11" t="str">
+        <f aca="false">IF(E21="","",IF(E21&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I21" s="11"/>
       <c r="J21" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2481,7 +2561,10 @@
       <c r="E22" s="11"/>
       <c r="F22" s="11"/>
       <c r="G22" s="13"/>
-      <c r="H22" s="11"/>
+      <c r="H22" s="11" t="str">
+        <f aca="false">IF(E22="","",IF(E22&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I22" s="11"/>
       <c r="J22" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2534,7 +2617,10 @@
       <c r="E23" s="11"/>
       <c r="F23" s="11"/>
       <c r="G23" s="13"/>
-      <c r="H23" s="11"/>
+      <c r="H23" s="11" t="str">
+        <f aca="false">IF(E23="","",IF(E23&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I23" s="11"/>
       <c r="J23" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2587,7 +2673,10 @@
       <c r="E24" s="11"/>
       <c r="F24" s="11"/>
       <c r="G24" s="13"/>
-      <c r="H24" s="11"/>
+      <c r="H24" s="11" t="str">
+        <f aca="false">IF(E24="","",IF(E24&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I24" s="11"/>
       <c r="J24" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2640,7 +2729,10 @@
       <c r="E25" s="11"/>
       <c r="F25" s="11"/>
       <c r="G25" s="13"/>
-      <c r="H25" s="11"/>
+      <c r="H25" s="11" t="str">
+        <f aca="false">IF(E25="","",IF(E25&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I25" s="11"/>
       <c r="J25" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2693,7 +2785,10 @@
       <c r="E26" s="11"/>
       <c r="F26" s="11"/>
       <c r="G26" s="13"/>
-      <c r="H26" s="11"/>
+      <c r="H26" s="11" t="str">
+        <f aca="false">IF(E26="","",IF(E26&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I26" s="11"/>
       <c r="J26" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2746,7 +2841,10 @@
       <c r="E27" s="11"/>
       <c r="F27" s="11"/>
       <c r="G27" s="13"/>
-      <c r="H27" s="11"/>
+      <c r="H27" s="11" t="str">
+        <f aca="false">IF(E27="","",IF(E27&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I27" s="11"/>
       <c r="J27" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2799,7 +2897,10 @@
       <c r="E28" s="11"/>
       <c r="F28" s="11"/>
       <c r="G28" s="13"/>
-      <c r="H28" s="11"/>
+      <c r="H28" s="11" t="str">
+        <f aca="false">IF(E28="","",IF(E28&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I28" s="11"/>
       <c r="J28" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2852,7 +2953,10 @@
       <c r="E29" s="11"/>
       <c r="F29" s="11"/>
       <c r="G29" s="13"/>
-      <c r="H29" s="11"/>
+      <c r="H29" s="11" t="str">
+        <f aca="false">IF(E29="","",IF(E29&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I29" s="11"/>
       <c r="J29" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2905,7 +3009,10 @@
       <c r="E30" s="11"/>
       <c r="F30" s="11"/>
       <c r="G30" s="13"/>
-      <c r="H30" s="11"/>
+      <c r="H30" s="11" t="str">
+        <f aca="false">IF(E30="","",IF(E30&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I30" s="11"/>
       <c r="J30" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -2958,7 +3065,10 @@
       <c r="E31" s="11"/>
       <c r="F31" s="11"/>
       <c r="G31" s="13"/>
-      <c r="H31" s="11"/>
+      <c r="H31" s="11" t="str">
+        <f aca="false">IF(E31="","",IF(E31&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I31" s="11"/>
       <c r="J31" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -3011,7 +3121,10 @@
       <c r="E32" s="11"/>
       <c r="F32" s="11"/>
       <c r="G32" s="13"/>
-      <c r="H32" s="11"/>
+      <c r="H32" s="11" t="str">
+        <f aca="false">IF(E32="","",IF(E32&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I32" s="11"/>
       <c r="J32" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -3064,7 +3177,10 @@
       <c r="E33" s="11"/>
       <c r="F33" s="11"/>
       <c r="G33" s="13"/>
-      <c r="H33" s="11"/>
+      <c r="H33" s="11" t="str">
+        <f aca="false">IF(E33="","",IF(E33&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I33" s="11"/>
       <c r="J33" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -3117,7 +3233,10 @@
       <c r="E34" s="11"/>
       <c r="F34" s="11"/>
       <c r="G34" s="13"/>
-      <c r="H34" s="11"/>
+      <c r="H34" s="11" t="str">
+        <f aca="false">IF(E34="","",IF(E34&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I34" s="11"/>
       <c r="J34" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -3170,7 +3289,10 @@
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
       <c r="G35" s="13"/>
-      <c r="H35" s="11"/>
+      <c r="H35" s="11" t="str">
+        <f aca="false">IF(E35="","",IF(E35&lt;Parametros!$B$24,Parametros!$B$23,0))</f>
+        <v/>
+      </c>
       <c r="I35" s="11"/>
       <c r="J35" s="11" t="n">
         <f aca="false">Parametros!$B$12</f>
@@ -3273,70 +3395,70 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D6" s="14" t="n">
         <v>10000</v>
@@ -4486,7 +4608,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="D36" s="20" t="n">
         <f aca="false">SUM(D6:D35)</f>
@@ -4573,55 +4695,55 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C6" s="14" t="n">
         <v>30</v>
@@ -5468,7 +5590,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="26" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="I37" s="21" t="n">
         <f aca="false">SUM(I6:I35)</f>
@@ -5477,7 +5599,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="26" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="I38" s="12" t="n">
         <f aca="false">Parametros!$B$16+Parametros!$B$21</f>
@@ -5486,7 +5608,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="26" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="I39" s="21" t="n">
         <f aca="false">I38-I37</f>
@@ -5526,17 +5648,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B3" s="11" t="n">
         <v>0</v>
@@ -5544,24 +5666,24 @@
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -5570,7 +5692,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="12" t="n">
@@ -5588,7 +5710,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
@@ -5597,7 +5719,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">Parametros!$B$11</f>
@@ -5618,7 +5740,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
@@ -5627,7 +5749,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B10" s="21" t="n">
         <f aca="false">B5-SUM(B6:B9)</f>
@@ -5648,7 +5770,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B11" s="21" t="n">
         <f aca="false">$B$3+B10</f>
@@ -5669,7 +5791,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
@@ -5678,7 +5800,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">B12</f>
@@ -5699,7 +5821,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">MAX(0,Parametros!$B$21-B13)</f>
@@ -5720,12 +5842,12 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -5758,34 +5880,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B5" s="14"/>
       <c r="C5" s="14"/>
@@ -5797,7 +5919,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
@@ -5809,7 +5931,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
@@ -5821,7 +5943,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
@@ -5833,7 +5955,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
@@ -5845,7 +5967,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
@@ -5857,7 +5979,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
@@ -5869,7 +5991,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">B6*Parametros!$B$4</f>
@@ -5890,7 +6012,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
@@ -5902,7 +6024,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B14" s="21" t="n">
         <f aca="false">B6-SUM(B7:B13)</f>
@@ -5923,7 +6045,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B15" s="17" t="str">
         <f aca="false">IF(B6&gt;0,B14/B6,"")</f>
@@ -5944,7 +6066,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B16" s="12" t="n">
         <f aca="false">Parametros!$B$11</f>
@@ -5965,7 +6087,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B17" s="21" t="n">
         <f aca="false">B14-B16</f>
@@ -5986,7 +6108,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">SUM($B17:B17)</f>
@@ -6007,7 +6129,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">Parametros!$B$7-B18</f>
@@ -6028,7 +6150,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B20" s="17" t="n">
         <f aca="false">IF(Parametros!$B$7&gt;0,B18/Parametros!$B$7,"")</f>
@@ -6049,7 +6171,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B21" s="12" t="str">
         <f aca="false">IF(B5&gt;0,B6/B5,"")</f>
@@ -6070,7 +6192,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B22" s="17" t="str">
         <f aca="false">IF(B6&gt;0,B13/B6,"")</f>
@@ -6091,7 +6213,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -6127,17 +6249,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="28" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B4" s="12" t="n">
         <f aca="false">Parametros!$B$7/Parametros!$B$8</f>
@@ -6146,7 +6268,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B5" s="12" t="n">
         <f aca="false">Parametros!$B$11</f>
@@ -6155,7 +6277,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="28" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B6" s="21" t="n">
         <f aca="false">B4+B5</f>
@@ -6164,7 +6286,7 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="29" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B7" s="12" t="n">
         <f aca="false">2*Parametros!$B$7/(Parametros!$B$8+1)</f>
@@ -6173,7 +6295,7 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="29" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B8" s="21" t="n">
         <f aca="false">B7+B5</f>
@@ -6182,25 +6304,25 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6292,7 +6414,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adapt spreadsheet to ML + Shopee with shared own stock
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W6G8eVwxeF9fr6fyaH3NLi
</commit_message>
<xml_diff>
--- a/central-loja/planilha_gestao_loja.xlsx
+++ b/central-loja/planilha_gestao_loja.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="190">
   <si>
     <t xml:space="preserve">Central de Gestão da Loja – Planilha base (v0.4)</t>
   </si>
@@ -56,7 +56,7 @@
     <t xml:space="preserve">Ads – dados do Mercado Ads exportados do Painel; calcula ACOS, ROAS, CPC, CTR, conversão e compara com o teto do SKU.</t>
   </si>
   <si>
-    <t xml:space="preserve">Estoque – cobertura em dias e ponto de reposição por SKU (você não usa ERP; esta é a fonte única de estoque).</t>
+    <t xml:space="preserve">Estoque – estoque próprio compartilhado (ML Coleta + Shopee) separado do Full; cobertura e ponto de reposição (sem ERP, esta é a fonte única).</t>
   </si>
   <si>
     <t xml:space="preserve">Fluxo_Caixa – boletos de compra (30 dias) x entradas do ML mês a mês: mostra se o lucro virou caixa.</t>
@@ -359,28 +359,46 @@
     <t xml:space="preserve">Campanha exemplo</t>
   </si>
   <si>
+    <t xml:space="preserve">ML</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">Estoque e reposição</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fonte única de estoque (sem ERP). Atualize semanalmente. Compra só com capital disponível e margem confirmada. Linha 6 = EXEMPLO ILUSTRATIVO (apagar).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estoque atual (un)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vendas últimos 30 dias (un)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Giro diário (un/dia)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cobertura (dias)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ponto de reposição (un)</t>
+    <t xml:space="preserve">Estoque e reposição (estoque próprio compartilhado: ML Coleta + Shopee)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fonte única de estoque (sem ERP). Atualize a cada venda nos dois canais para evitar venda sem estoque. O estoque no Full é do ML e não atende a Shopee. Linha 6 = EXEMPLO ILUSTRATIVO (apagar).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estoque próprio (un) – ML Coleta + Shopee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estoque no Full (un) – só ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vendas 30 dias – ML Full (un)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vendas 30 dias – ML Coleta (un)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vendas 30 dias – Shopee (un)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giro diário próprio (un/dia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giro diário Full (un/dia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobertura estoque próprio (dias)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobertura Full (dias)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto de reposição próprio (un)</t>
   </si>
   <si>
     <t xml:space="preserve">Custo unitário (R$)</t>
@@ -522,6 +540,18 @@
   </si>
   <si>
     <t xml:space="preserve">Atenção: meta = lucro contábil (receita menos todos os custos). Reposição de estoque não é descontada aqui; acompanhe o caixa separadamente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faturamento por canal (informativo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faturamento Mercado Livre (R$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faturamento Shopee (R$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diferença vs. faturamento bruto acima (deve ser zero)</t>
   </si>
   <si>
     <t xml:space="preserve">Simulador: pedidos necessários para a meta</t>
@@ -1187,7 +1217,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
@@ -3351,7 +3381,7 @@
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D6:D35" type="list">
-      <formula1>"Full,Coleta"</formula1>
+      <formula1>"Full,Coleta,Shopee"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M6:M35" type="list">
@@ -3374,7 +3404,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:P36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -3391,6 +3421,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3449,6 +3480,9 @@
       <c r="O5" s="5" t="s">
         <v>107</v>
       </c>
+      <c r="P5" s="5" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
@@ -3502,6 +3536,9 @@
       <c r="O6" s="6" t="str">
         <f aca="false">IF(F6="","",IF(AND(F6&gt;0,G6=0),"Gasto sem venda",IF(OR(L6="",N6=""),"Sem teto/ACOS",IF(L6&lt;=N6,"Dentro do teto","ACIMA do teto"))))</f>
         <v>Dentro do teto</v>
+      </c>
+      <c r="P6" s="16" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3541,6 +3578,7 @@
         <f aca="false">IF(F7="","",IF(AND(F7&gt;0,G7=0),"Gasto sem venda",IF(OR(L7="",N7=""),"Sem teto/ACOS",IF(L7&lt;=N7,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P7" s="16"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16"/>
@@ -3579,6 +3617,7 @@
         <f aca="false">IF(F8="","",IF(AND(F8&gt;0,G8=0),"Gasto sem venda",IF(OR(L8="",N8=""),"Sem teto/ACOS",IF(L8&lt;=N8,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16"/>
@@ -3617,6 +3656,7 @@
         <f aca="false">IF(F9="","",IF(AND(F9&gt;0,G9=0),"Gasto sem venda",IF(OR(L9="",N9=""),"Sem teto/ACOS",IF(L9&lt;=N9,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P9" s="16"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16"/>
@@ -3655,6 +3695,7 @@
         <f aca="false">IF(F10="","",IF(AND(F10&gt;0,G10=0),"Gasto sem venda",IF(OR(L10="",N10=""),"Sem teto/ACOS",IF(L10&lt;=N10,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P10" s="16"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16"/>
@@ -3693,6 +3734,7 @@
         <f aca="false">IF(F11="","",IF(AND(F11&gt;0,G11=0),"Gasto sem venda",IF(OR(L11="",N11=""),"Sem teto/ACOS",IF(L11&lt;=N11,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P11" s="16"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16"/>
@@ -3731,6 +3773,7 @@
         <f aca="false">IF(F12="","",IF(AND(F12&gt;0,G12=0),"Gasto sem venda",IF(OR(L12="",N12=""),"Sem teto/ACOS",IF(L12&lt;=N12,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P12" s="16"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16"/>
@@ -3769,6 +3812,7 @@
         <f aca="false">IF(F13="","",IF(AND(F13&gt;0,G13=0),"Gasto sem venda",IF(OR(L13="",N13=""),"Sem teto/ACOS",IF(L13&lt;=N13,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P13" s="16"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16"/>
@@ -3807,6 +3851,7 @@
         <f aca="false">IF(F14="","",IF(AND(F14&gt;0,G14=0),"Gasto sem venda",IF(OR(L14="",N14=""),"Sem teto/ACOS",IF(L14&lt;=N14,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P14" s="16"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16"/>
@@ -3845,6 +3890,7 @@
         <f aca="false">IF(F15="","",IF(AND(F15&gt;0,G15=0),"Gasto sem venda",IF(OR(L15="",N15=""),"Sem teto/ACOS",IF(L15&lt;=N15,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P15" s="16"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16"/>
@@ -3883,6 +3929,7 @@
         <f aca="false">IF(F16="","",IF(AND(F16&gt;0,G16=0),"Gasto sem venda",IF(OR(L16="",N16=""),"Sem teto/ACOS",IF(L16&lt;=N16,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P16" s="16"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="16"/>
@@ -3921,6 +3968,7 @@
         <f aca="false">IF(F17="","",IF(AND(F17&gt;0,G17=0),"Gasto sem venda",IF(OR(L17="",N17=""),"Sem teto/ACOS",IF(L17&lt;=N17,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P17" s="16"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16"/>
@@ -3959,6 +4007,7 @@
         <f aca="false">IF(F18="","",IF(AND(F18&gt;0,G18=0),"Gasto sem venda",IF(OR(L18="",N18=""),"Sem teto/ACOS",IF(L18&lt;=N18,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P18" s="16"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="16"/>
@@ -3997,6 +4046,7 @@
         <f aca="false">IF(F19="","",IF(AND(F19&gt;0,G19=0),"Gasto sem venda",IF(OR(L19="",N19=""),"Sem teto/ACOS",IF(L19&lt;=N19,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P19" s="16"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16"/>
@@ -4035,6 +4085,7 @@
         <f aca="false">IF(F20="","",IF(AND(F20&gt;0,G20=0),"Gasto sem venda",IF(OR(L20="",N20=""),"Sem teto/ACOS",IF(L20&lt;=N20,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P20" s="16"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16"/>
@@ -4073,6 +4124,7 @@
         <f aca="false">IF(F21="","",IF(AND(F21&gt;0,G21=0),"Gasto sem venda",IF(OR(L21="",N21=""),"Sem teto/ACOS",IF(L21&lt;=N21,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P21" s="16"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16"/>
@@ -4111,6 +4163,7 @@
         <f aca="false">IF(F22="","",IF(AND(F22&gt;0,G22=0),"Gasto sem venda",IF(OR(L22="",N22=""),"Sem teto/ACOS",IF(L22&lt;=N22,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P22" s="16"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="16"/>
@@ -4149,6 +4202,7 @@
         <f aca="false">IF(F23="","",IF(AND(F23&gt;0,G23=0),"Gasto sem venda",IF(OR(L23="",N23=""),"Sem teto/ACOS",IF(L23&lt;=N23,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P23" s="16"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="16"/>
@@ -4187,6 +4241,7 @@
         <f aca="false">IF(F24="","",IF(AND(F24&gt;0,G24=0),"Gasto sem venda",IF(OR(L24="",N24=""),"Sem teto/ACOS",IF(L24&lt;=N24,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P24" s="16"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16"/>
@@ -4225,6 +4280,7 @@
         <f aca="false">IF(F25="","",IF(AND(F25&gt;0,G25=0),"Gasto sem venda",IF(OR(L25="",N25=""),"Sem teto/ACOS",IF(L25&lt;=N25,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P25" s="16"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16"/>
@@ -4263,6 +4319,7 @@
         <f aca="false">IF(F26="","",IF(AND(F26&gt;0,G26=0),"Gasto sem venda",IF(OR(L26="",N26=""),"Sem teto/ACOS",IF(L26&lt;=N26,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P26" s="16"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="16"/>
@@ -4301,6 +4358,7 @@
         <f aca="false">IF(F27="","",IF(AND(F27&gt;0,G27=0),"Gasto sem venda",IF(OR(L27="",N27=""),"Sem teto/ACOS",IF(L27&lt;=N27,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P27" s="16"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16"/>
@@ -4339,6 +4397,7 @@
         <f aca="false">IF(F28="","",IF(AND(F28&gt;0,G28=0),"Gasto sem venda",IF(OR(L28="",N28=""),"Sem teto/ACOS",IF(L28&lt;=N28,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P28" s="16"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16"/>
@@ -4377,6 +4436,7 @@
         <f aca="false">IF(F29="","",IF(AND(F29&gt;0,G29=0),"Gasto sem venda",IF(OR(L29="",N29=""),"Sem teto/ACOS",IF(L29&lt;=N29,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P29" s="16"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16"/>
@@ -4415,6 +4475,7 @@
         <f aca="false">IF(F30="","",IF(AND(F30&gt;0,G30=0),"Gasto sem venda",IF(OR(L30="",N30=""),"Sem teto/ACOS",IF(L30&lt;=N30,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P30" s="16"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="16"/>
@@ -4453,6 +4514,7 @@
         <f aca="false">IF(F31="","",IF(AND(F31&gt;0,G31=0),"Gasto sem venda",IF(OR(L31="",N31=""),"Sem teto/ACOS",IF(L31&lt;=N31,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P31" s="16"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16"/>
@@ -4491,6 +4553,7 @@
         <f aca="false">IF(F32="","",IF(AND(F32&gt;0,G32=0),"Gasto sem venda",IF(OR(L32="",N32=""),"Sem teto/ACOS",IF(L32&lt;=N32,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P32" s="16"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16"/>
@@ -4529,6 +4592,7 @@
         <f aca="false">IF(F33="","",IF(AND(F33&gt;0,G33=0),"Gasto sem venda",IF(OR(L33="",N33=""),"Sem teto/ACOS",IF(L33&lt;=N33,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P33" s="16"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="16"/>
@@ -4567,6 +4631,7 @@
         <f aca="false">IF(F34="","",IF(AND(F34&gt;0,G34=0),"Gasto sem venda",IF(OR(L34="",N34=""),"Sem teto/ACOS",IF(L34&lt;=N34,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P34" s="16"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16"/>
@@ -4605,10 +4670,11 @@
         <f aca="false">IF(F35="","",IF(AND(F35&gt;0,G35=0),"Gasto sem venda",IF(OR(L35="",N35=""),"Sem teto/ACOS",IF(L35&lt;=N35,"Dentro do teto","ACIMA do teto"))))</f>
         <v/>
       </c>
+      <c r="P35" s="16"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D36" s="20" t="n">
         <f aca="false">SUM(D6:D35)</f>
@@ -4663,6 +4729,12 @@
       <formula>"Dentro do teto"</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P6:P35" type="list">
+      <formula1>"ML,Shopee"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4678,29 +4750,31 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:O39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4708,917 +4782,1233 @@
         <v>65</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>68</v>
+        <v>114</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J5" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="N5" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="K5" s="5" t="s">
-        <v>120</v>
+      <c r="O5" s="5" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>89</v>
+      <c r="B6" s="14" t="n">
+        <v>30</v>
       </c>
       <c r="C6" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="G6" s="18" t="n">
+        <f aca="false">IF(A6="","",(E6+F6)/30)</f>
+        <v>1</v>
+      </c>
+      <c r="H6" s="18" t="n">
+        <f aca="false">IF(A6="","",D6/30)</f>
+        <v>0.333333333333333</v>
+      </c>
+      <c r="I6" s="24" t="n">
+        <f aca="false">IF(A6="","",IF(G6&gt;0,B6/G6,""))</f>
         <v>30</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="J6" s="24" t="n">
+        <f aca="false">IF(A6="","",IF(H6&gt;0,C6/H6,""))</f>
         <v>30</v>
       </c>
-      <c r="E6" s="18" t="n">
-        <f aca="false">IF(A6="","",D6/30)</f>
-        <v>1</v>
-      </c>
-      <c r="F6" s="24" t="n">
-        <f aca="false">IF(A6="","",IF(E6&gt;0,C6/E6,"sem giro"))</f>
-        <v>30</v>
-      </c>
-      <c r="G6" s="24" t="n">
-        <f aca="false">IF(A6="","",E6*(Parametros!$B$17+Parametros!$B$19))</f>
+      <c r="K6" s="24" t="n">
+        <f aca="false">IF(A6="","",G6*(Parametros!$B$17+Parametros!$B$19))</f>
         <v>35</v>
       </c>
-      <c r="H6" s="11" t="n">
+      <c r="L6" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="I6" s="12" t="n">
-        <f aca="false">IF(A6="","",E6*30*H6)</f>
-        <v>1200</v>
-      </c>
-      <c r="J6" s="6" t="str">
-        <f aca="false">IF(A6="","",IF(C6&lt;=0,"RUPTURA",IF(F6="sem giro","Sem giro: revisar",IF(C6&lt;=G6,"REPOR (abaixo do ponto)",IF(F6&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
+      <c r="M6" s="12" t="n">
+        <f aca="false">IF(A6="","",(G6+H6)*30*L6)</f>
+        <v>1600</v>
+      </c>
+      <c r="N6" s="6" t="str">
+        <f aca="false">IF(A6="","",IF(OR(AND(G6&gt;0,B6&lt;=0),AND(H6&gt;0,C6&lt;=0)),"RUPTURA",IF(OR(AND(G6&gt;0,B6&lt;=K6),AND(H6&gt;0,C6&lt;=H6*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G6+H6=0,"Sem giro: revisar",IF(OR(AND(G6&gt;0,I6&gt;120),AND(H6&gt;0,J6&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
         <v>REPOR (abaixo do ponto)</v>
       </c>
-      <c r="K6" s="25"/>
+      <c r="O6" s="25"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16"/>
-      <c r="B7" s="16"/>
+      <c r="B7" s="14"/>
       <c r="C7" s="14"/>
       <c r="D7" s="14"/>
-      <c r="E7" s="18" t="str">
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="18" t="str">
+        <f aca="false">IF(A7="","",(E7+F7)/30)</f>
+        <v/>
+      </c>
+      <c r="H7" s="18" t="str">
         <f aca="false">IF(A7="","",D7/30)</f>
         <v/>
       </c>
-      <c r="F7" s="24" t="str">
-        <f aca="false">IF(A7="","",IF(E7&gt;0,C7/E7,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G7" s="24" t="str">
-        <f aca="false">IF(A7="","",E7*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H7" s="11"/>
-      <c r="I7" s="12" t="str">
-        <f aca="false">IF(A7="","",E7*30*H7)</f>
-        <v/>
-      </c>
-      <c r="J7" s="6" t="str">
-        <f aca="false">IF(A7="","",IF(C7&lt;=0,"RUPTURA",IF(F7="sem giro","Sem giro: revisar",IF(C7&lt;=G7,"REPOR (abaixo do ponto)",IF(F7&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K7" s="25"/>
+      <c r="I7" s="24" t="str">
+        <f aca="false">IF(A7="","",IF(G7&gt;0,B7/G7,""))</f>
+        <v/>
+      </c>
+      <c r="J7" s="24" t="str">
+        <f aca="false">IF(A7="","",IF(H7&gt;0,C7/H7,""))</f>
+        <v/>
+      </c>
+      <c r="K7" s="24" t="str">
+        <f aca="false">IF(A7="","",G7*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L7" s="11"/>
+      <c r="M7" s="12" t="str">
+        <f aca="false">IF(A7="","",(G7+H7)*30*L7)</f>
+        <v/>
+      </c>
+      <c r="N7" s="6" t="str">
+        <f aca="false">IF(A7="","",IF(OR(AND(G7&gt;0,B7&lt;=0),AND(H7&gt;0,C7&lt;=0)),"RUPTURA",IF(OR(AND(G7&gt;0,B7&lt;=K7),AND(H7&gt;0,C7&lt;=H7*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G7+H7=0,"Sem giro: revisar",IF(OR(AND(G7&gt;0,I7&gt;120),AND(H7&gt;0,J7&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O7" s="25"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16"/>
-      <c r="B8" s="16"/>
+      <c r="B8" s="14"/>
       <c r="C8" s="14"/>
       <c r="D8" s="14"/>
-      <c r="E8" s="18" t="str">
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="18" t="str">
+        <f aca="false">IF(A8="","",(E8+F8)/30)</f>
+        <v/>
+      </c>
+      <c r="H8" s="18" t="str">
         <f aca="false">IF(A8="","",D8/30)</f>
         <v/>
       </c>
-      <c r="F8" s="24" t="str">
-        <f aca="false">IF(A8="","",IF(E8&gt;0,C8/E8,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G8" s="24" t="str">
-        <f aca="false">IF(A8="","",E8*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H8" s="11"/>
-      <c r="I8" s="12" t="str">
-        <f aca="false">IF(A8="","",E8*30*H8)</f>
-        <v/>
-      </c>
-      <c r="J8" s="6" t="str">
-        <f aca="false">IF(A8="","",IF(C8&lt;=0,"RUPTURA",IF(F8="sem giro","Sem giro: revisar",IF(C8&lt;=G8,"REPOR (abaixo do ponto)",IF(F8&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K8" s="25"/>
+      <c r="I8" s="24" t="str">
+        <f aca="false">IF(A8="","",IF(G8&gt;0,B8/G8,""))</f>
+        <v/>
+      </c>
+      <c r="J8" s="24" t="str">
+        <f aca="false">IF(A8="","",IF(H8&gt;0,C8/H8,""))</f>
+        <v/>
+      </c>
+      <c r="K8" s="24" t="str">
+        <f aca="false">IF(A8="","",G8*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L8" s="11"/>
+      <c r="M8" s="12" t="str">
+        <f aca="false">IF(A8="","",(G8+H8)*30*L8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="6" t="str">
+        <f aca="false">IF(A8="","",IF(OR(AND(G8&gt;0,B8&lt;=0),AND(H8&gt;0,C8&lt;=0)),"RUPTURA",IF(OR(AND(G8&gt;0,B8&lt;=K8),AND(H8&gt;0,C8&lt;=H8*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G8+H8=0,"Sem giro: revisar",IF(OR(AND(G8&gt;0,I8&gt;120),AND(H8&gt;0,J8&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O8" s="25"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16"/>
-      <c r="B9" s="16"/>
+      <c r="B9" s="14"/>
       <c r="C9" s="14"/>
       <c r="D9" s="14"/>
-      <c r="E9" s="18" t="str">
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="18" t="str">
+        <f aca="false">IF(A9="","",(E9+F9)/30)</f>
+        <v/>
+      </c>
+      <c r="H9" s="18" t="str">
         <f aca="false">IF(A9="","",D9/30)</f>
         <v/>
       </c>
-      <c r="F9" s="24" t="str">
-        <f aca="false">IF(A9="","",IF(E9&gt;0,C9/E9,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G9" s="24" t="str">
-        <f aca="false">IF(A9="","",E9*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H9" s="11"/>
-      <c r="I9" s="12" t="str">
-        <f aca="false">IF(A9="","",E9*30*H9)</f>
-        <v/>
-      </c>
-      <c r="J9" s="6" t="str">
-        <f aca="false">IF(A9="","",IF(C9&lt;=0,"RUPTURA",IF(F9="sem giro","Sem giro: revisar",IF(C9&lt;=G9,"REPOR (abaixo do ponto)",IF(F9&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K9" s="25"/>
+      <c r="I9" s="24" t="str">
+        <f aca="false">IF(A9="","",IF(G9&gt;0,B9/G9,""))</f>
+        <v/>
+      </c>
+      <c r="J9" s="24" t="str">
+        <f aca="false">IF(A9="","",IF(H9&gt;0,C9/H9,""))</f>
+        <v/>
+      </c>
+      <c r="K9" s="24" t="str">
+        <f aca="false">IF(A9="","",G9*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L9" s="11"/>
+      <c r="M9" s="12" t="str">
+        <f aca="false">IF(A9="","",(G9+H9)*30*L9)</f>
+        <v/>
+      </c>
+      <c r="N9" s="6" t="str">
+        <f aca="false">IF(A9="","",IF(OR(AND(G9&gt;0,B9&lt;=0),AND(H9&gt;0,C9&lt;=0)),"RUPTURA",IF(OR(AND(G9&gt;0,B9&lt;=K9),AND(H9&gt;0,C9&lt;=H9*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G9+H9=0,"Sem giro: revisar",IF(OR(AND(G9&gt;0,I9&gt;120),AND(H9&gt;0,J9&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O9" s="25"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16"/>
-      <c r="B10" s="16"/>
+      <c r="B10" s="14"/>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
-      <c r="E10" s="18" t="str">
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="18" t="str">
+        <f aca="false">IF(A10="","",(E10+F10)/30)</f>
+        <v/>
+      </c>
+      <c r="H10" s="18" t="str">
         <f aca="false">IF(A10="","",D10/30)</f>
         <v/>
       </c>
-      <c r="F10" s="24" t="str">
-        <f aca="false">IF(A10="","",IF(E10&gt;0,C10/E10,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G10" s="24" t="str">
-        <f aca="false">IF(A10="","",E10*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H10" s="11"/>
-      <c r="I10" s="12" t="str">
-        <f aca="false">IF(A10="","",E10*30*H10)</f>
-        <v/>
-      </c>
-      <c r="J10" s="6" t="str">
-        <f aca="false">IF(A10="","",IF(C10&lt;=0,"RUPTURA",IF(F10="sem giro","Sem giro: revisar",IF(C10&lt;=G10,"REPOR (abaixo do ponto)",IF(F10&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K10" s="25"/>
+      <c r="I10" s="24" t="str">
+        <f aca="false">IF(A10="","",IF(G10&gt;0,B10/G10,""))</f>
+        <v/>
+      </c>
+      <c r="J10" s="24" t="str">
+        <f aca="false">IF(A10="","",IF(H10&gt;0,C10/H10,""))</f>
+        <v/>
+      </c>
+      <c r="K10" s="24" t="str">
+        <f aca="false">IF(A10="","",G10*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L10" s="11"/>
+      <c r="M10" s="12" t="str">
+        <f aca="false">IF(A10="","",(G10+H10)*30*L10)</f>
+        <v/>
+      </c>
+      <c r="N10" s="6" t="str">
+        <f aca="false">IF(A10="","",IF(OR(AND(G10&gt;0,B10&lt;=0),AND(H10&gt;0,C10&lt;=0)),"RUPTURA",IF(OR(AND(G10&gt;0,B10&lt;=K10),AND(H10&gt;0,C10&lt;=H10*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G10+H10=0,"Sem giro: revisar",IF(OR(AND(G10&gt;0,I10&gt;120),AND(H10&gt;0,J10&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O10" s="25"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16"/>
-      <c r="B11" s="16"/>
+      <c r="B11" s="14"/>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
-      <c r="E11" s="18" t="str">
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="18" t="str">
+        <f aca="false">IF(A11="","",(E11+F11)/30)</f>
+        <v/>
+      </c>
+      <c r="H11" s="18" t="str">
         <f aca="false">IF(A11="","",D11/30)</f>
         <v/>
       </c>
-      <c r="F11" s="24" t="str">
-        <f aca="false">IF(A11="","",IF(E11&gt;0,C11/E11,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G11" s="24" t="str">
-        <f aca="false">IF(A11="","",E11*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H11" s="11"/>
-      <c r="I11" s="12" t="str">
-        <f aca="false">IF(A11="","",E11*30*H11)</f>
-        <v/>
-      </c>
-      <c r="J11" s="6" t="str">
-        <f aca="false">IF(A11="","",IF(C11&lt;=0,"RUPTURA",IF(F11="sem giro","Sem giro: revisar",IF(C11&lt;=G11,"REPOR (abaixo do ponto)",IF(F11&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K11" s="25"/>
+      <c r="I11" s="24" t="str">
+        <f aca="false">IF(A11="","",IF(G11&gt;0,B11/G11,""))</f>
+        <v/>
+      </c>
+      <c r="J11" s="24" t="str">
+        <f aca="false">IF(A11="","",IF(H11&gt;0,C11/H11,""))</f>
+        <v/>
+      </c>
+      <c r="K11" s="24" t="str">
+        <f aca="false">IF(A11="","",G11*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L11" s="11"/>
+      <c r="M11" s="12" t="str">
+        <f aca="false">IF(A11="","",(G11+H11)*30*L11)</f>
+        <v/>
+      </c>
+      <c r="N11" s="6" t="str">
+        <f aca="false">IF(A11="","",IF(OR(AND(G11&gt;0,B11&lt;=0),AND(H11&gt;0,C11&lt;=0)),"RUPTURA",IF(OR(AND(G11&gt;0,B11&lt;=K11),AND(H11&gt;0,C11&lt;=H11*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G11+H11=0,"Sem giro: revisar",IF(OR(AND(G11&gt;0,I11&gt;120),AND(H11&gt;0,J11&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O11" s="25"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16"/>
-      <c r="B12" s="16"/>
+      <c r="B12" s="14"/>
       <c r="C12" s="14"/>
       <c r="D12" s="14"/>
-      <c r="E12" s="18" t="str">
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="18" t="str">
+        <f aca="false">IF(A12="","",(E12+F12)/30)</f>
+        <v/>
+      </c>
+      <c r="H12" s="18" t="str">
         <f aca="false">IF(A12="","",D12/30)</f>
         <v/>
       </c>
-      <c r="F12" s="24" t="str">
-        <f aca="false">IF(A12="","",IF(E12&gt;0,C12/E12,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G12" s="24" t="str">
-        <f aca="false">IF(A12="","",E12*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H12" s="11"/>
-      <c r="I12" s="12" t="str">
-        <f aca="false">IF(A12="","",E12*30*H12)</f>
-        <v/>
-      </c>
-      <c r="J12" s="6" t="str">
-        <f aca="false">IF(A12="","",IF(C12&lt;=0,"RUPTURA",IF(F12="sem giro","Sem giro: revisar",IF(C12&lt;=G12,"REPOR (abaixo do ponto)",IF(F12&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K12" s="25"/>
+      <c r="I12" s="24" t="str">
+        <f aca="false">IF(A12="","",IF(G12&gt;0,B12/G12,""))</f>
+        <v/>
+      </c>
+      <c r="J12" s="24" t="str">
+        <f aca="false">IF(A12="","",IF(H12&gt;0,C12/H12,""))</f>
+        <v/>
+      </c>
+      <c r="K12" s="24" t="str">
+        <f aca="false">IF(A12="","",G12*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L12" s="11"/>
+      <c r="M12" s="12" t="str">
+        <f aca="false">IF(A12="","",(G12+H12)*30*L12)</f>
+        <v/>
+      </c>
+      <c r="N12" s="6" t="str">
+        <f aca="false">IF(A12="","",IF(OR(AND(G12&gt;0,B12&lt;=0),AND(H12&gt;0,C12&lt;=0)),"RUPTURA",IF(OR(AND(G12&gt;0,B12&lt;=K12),AND(H12&gt;0,C12&lt;=H12*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G12+H12=0,"Sem giro: revisar",IF(OR(AND(G12&gt;0,I12&gt;120),AND(H12&gt;0,J12&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O12" s="25"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16"/>
-      <c r="B13" s="16"/>
+      <c r="B13" s="14"/>
       <c r="C13" s="14"/>
       <c r="D13" s="14"/>
-      <c r="E13" s="18" t="str">
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="18" t="str">
+        <f aca="false">IF(A13="","",(E13+F13)/30)</f>
+        <v/>
+      </c>
+      <c r="H13" s="18" t="str">
         <f aca="false">IF(A13="","",D13/30)</f>
         <v/>
       </c>
-      <c r="F13" s="24" t="str">
-        <f aca="false">IF(A13="","",IF(E13&gt;0,C13/E13,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G13" s="24" t="str">
-        <f aca="false">IF(A13="","",E13*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H13" s="11"/>
-      <c r="I13" s="12" t="str">
-        <f aca="false">IF(A13="","",E13*30*H13)</f>
-        <v/>
-      </c>
-      <c r="J13" s="6" t="str">
-        <f aca="false">IF(A13="","",IF(C13&lt;=0,"RUPTURA",IF(F13="sem giro","Sem giro: revisar",IF(C13&lt;=G13,"REPOR (abaixo do ponto)",IF(F13&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K13" s="25"/>
+      <c r="I13" s="24" t="str">
+        <f aca="false">IF(A13="","",IF(G13&gt;0,B13/G13,""))</f>
+        <v/>
+      </c>
+      <c r="J13" s="24" t="str">
+        <f aca="false">IF(A13="","",IF(H13&gt;0,C13/H13,""))</f>
+        <v/>
+      </c>
+      <c r="K13" s="24" t="str">
+        <f aca="false">IF(A13="","",G13*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L13" s="11"/>
+      <c r="M13" s="12" t="str">
+        <f aca="false">IF(A13="","",(G13+H13)*30*L13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="6" t="str">
+        <f aca="false">IF(A13="","",IF(OR(AND(G13&gt;0,B13&lt;=0),AND(H13&gt;0,C13&lt;=0)),"RUPTURA",IF(OR(AND(G13&gt;0,B13&lt;=K13),AND(H13&gt;0,C13&lt;=H13*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G13+H13=0,"Sem giro: revisar",IF(OR(AND(G13&gt;0,I13&gt;120),AND(H13&gt;0,J13&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O13" s="25"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16"/>
-      <c r="B14" s="16"/>
+      <c r="B14" s="14"/>
       <c r="C14" s="14"/>
       <c r="D14" s="14"/>
-      <c r="E14" s="18" t="str">
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="18" t="str">
+        <f aca="false">IF(A14="","",(E14+F14)/30)</f>
+        <v/>
+      </c>
+      <c r="H14" s="18" t="str">
         <f aca="false">IF(A14="","",D14/30)</f>
         <v/>
       </c>
-      <c r="F14" s="24" t="str">
-        <f aca="false">IF(A14="","",IF(E14&gt;0,C14/E14,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G14" s="24" t="str">
-        <f aca="false">IF(A14="","",E14*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H14" s="11"/>
-      <c r="I14" s="12" t="str">
-        <f aca="false">IF(A14="","",E14*30*H14)</f>
-        <v/>
-      </c>
-      <c r="J14" s="6" t="str">
-        <f aca="false">IF(A14="","",IF(C14&lt;=0,"RUPTURA",IF(F14="sem giro","Sem giro: revisar",IF(C14&lt;=G14,"REPOR (abaixo do ponto)",IF(F14&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K14" s="25"/>
+      <c r="I14" s="24" t="str">
+        <f aca="false">IF(A14="","",IF(G14&gt;0,B14/G14,""))</f>
+        <v/>
+      </c>
+      <c r="J14" s="24" t="str">
+        <f aca="false">IF(A14="","",IF(H14&gt;0,C14/H14,""))</f>
+        <v/>
+      </c>
+      <c r="K14" s="24" t="str">
+        <f aca="false">IF(A14="","",G14*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L14" s="11"/>
+      <c r="M14" s="12" t="str">
+        <f aca="false">IF(A14="","",(G14+H14)*30*L14)</f>
+        <v/>
+      </c>
+      <c r="N14" s="6" t="str">
+        <f aca="false">IF(A14="","",IF(OR(AND(G14&gt;0,B14&lt;=0),AND(H14&gt;0,C14&lt;=0)),"RUPTURA",IF(OR(AND(G14&gt;0,B14&lt;=K14),AND(H14&gt;0,C14&lt;=H14*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G14+H14=0,"Sem giro: revisar",IF(OR(AND(G14&gt;0,I14&gt;120),AND(H14&gt;0,J14&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O14" s="25"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16"/>
-      <c r="B15" s="16"/>
+      <c r="B15" s="14"/>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
-      <c r="E15" s="18" t="str">
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="18" t="str">
+        <f aca="false">IF(A15="","",(E15+F15)/30)</f>
+        <v/>
+      </c>
+      <c r="H15" s="18" t="str">
         <f aca="false">IF(A15="","",D15/30)</f>
         <v/>
       </c>
-      <c r="F15" s="24" t="str">
-        <f aca="false">IF(A15="","",IF(E15&gt;0,C15/E15,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G15" s="24" t="str">
-        <f aca="false">IF(A15="","",E15*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H15" s="11"/>
-      <c r="I15" s="12" t="str">
-        <f aca="false">IF(A15="","",E15*30*H15)</f>
-        <v/>
-      </c>
-      <c r="J15" s="6" t="str">
-        <f aca="false">IF(A15="","",IF(C15&lt;=0,"RUPTURA",IF(F15="sem giro","Sem giro: revisar",IF(C15&lt;=G15,"REPOR (abaixo do ponto)",IF(F15&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K15" s="25"/>
+      <c r="I15" s="24" t="str">
+        <f aca="false">IF(A15="","",IF(G15&gt;0,B15/G15,""))</f>
+        <v/>
+      </c>
+      <c r="J15" s="24" t="str">
+        <f aca="false">IF(A15="","",IF(H15&gt;0,C15/H15,""))</f>
+        <v/>
+      </c>
+      <c r="K15" s="24" t="str">
+        <f aca="false">IF(A15="","",G15*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L15" s="11"/>
+      <c r="M15" s="12" t="str">
+        <f aca="false">IF(A15="","",(G15+H15)*30*L15)</f>
+        <v/>
+      </c>
+      <c r="N15" s="6" t="str">
+        <f aca="false">IF(A15="","",IF(OR(AND(G15&gt;0,B15&lt;=0),AND(H15&gt;0,C15&lt;=0)),"RUPTURA",IF(OR(AND(G15&gt;0,B15&lt;=K15),AND(H15&gt;0,C15&lt;=H15*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G15+H15=0,"Sem giro: revisar",IF(OR(AND(G15&gt;0,I15&gt;120),AND(H15&gt;0,J15&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O15" s="25"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16"/>
-      <c r="B16" s="16"/>
+      <c r="B16" s="14"/>
       <c r="C16" s="14"/>
       <c r="D16" s="14"/>
-      <c r="E16" s="18" t="str">
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="18" t="str">
+        <f aca="false">IF(A16="","",(E16+F16)/30)</f>
+        <v/>
+      </c>
+      <c r="H16" s="18" t="str">
         <f aca="false">IF(A16="","",D16/30)</f>
         <v/>
       </c>
-      <c r="F16" s="24" t="str">
-        <f aca="false">IF(A16="","",IF(E16&gt;0,C16/E16,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G16" s="24" t="str">
-        <f aca="false">IF(A16="","",E16*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H16" s="11"/>
-      <c r="I16" s="12" t="str">
-        <f aca="false">IF(A16="","",E16*30*H16)</f>
-        <v/>
-      </c>
-      <c r="J16" s="6" t="str">
-        <f aca="false">IF(A16="","",IF(C16&lt;=0,"RUPTURA",IF(F16="sem giro","Sem giro: revisar",IF(C16&lt;=G16,"REPOR (abaixo do ponto)",IF(F16&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K16" s="25"/>
+      <c r="I16" s="24" t="str">
+        <f aca="false">IF(A16="","",IF(G16&gt;0,B16/G16,""))</f>
+        <v/>
+      </c>
+      <c r="J16" s="24" t="str">
+        <f aca="false">IF(A16="","",IF(H16&gt;0,C16/H16,""))</f>
+        <v/>
+      </c>
+      <c r="K16" s="24" t="str">
+        <f aca="false">IF(A16="","",G16*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L16" s="11"/>
+      <c r="M16" s="12" t="str">
+        <f aca="false">IF(A16="","",(G16+H16)*30*L16)</f>
+        <v/>
+      </c>
+      <c r="N16" s="6" t="str">
+        <f aca="false">IF(A16="","",IF(OR(AND(G16&gt;0,B16&lt;=0),AND(H16&gt;0,C16&lt;=0)),"RUPTURA",IF(OR(AND(G16&gt;0,B16&lt;=K16),AND(H16&gt;0,C16&lt;=H16*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G16+H16=0,"Sem giro: revisar",IF(OR(AND(G16&gt;0,I16&gt;120),AND(H16&gt;0,J16&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O16" s="25"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="16"/>
-      <c r="B17" s="16"/>
+      <c r="B17" s="14"/>
       <c r="C17" s="14"/>
       <c r="D17" s="14"/>
-      <c r="E17" s="18" t="str">
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="18" t="str">
+        <f aca="false">IF(A17="","",(E17+F17)/30)</f>
+        <v/>
+      </c>
+      <c r="H17" s="18" t="str">
         <f aca="false">IF(A17="","",D17/30)</f>
         <v/>
       </c>
-      <c r="F17" s="24" t="str">
-        <f aca="false">IF(A17="","",IF(E17&gt;0,C17/E17,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G17" s="24" t="str">
-        <f aca="false">IF(A17="","",E17*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H17" s="11"/>
-      <c r="I17" s="12" t="str">
-        <f aca="false">IF(A17="","",E17*30*H17)</f>
-        <v/>
-      </c>
-      <c r="J17" s="6" t="str">
-        <f aca="false">IF(A17="","",IF(C17&lt;=0,"RUPTURA",IF(F17="sem giro","Sem giro: revisar",IF(C17&lt;=G17,"REPOR (abaixo do ponto)",IF(F17&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K17" s="25"/>
+      <c r="I17" s="24" t="str">
+        <f aca="false">IF(A17="","",IF(G17&gt;0,B17/G17,""))</f>
+        <v/>
+      </c>
+      <c r="J17" s="24" t="str">
+        <f aca="false">IF(A17="","",IF(H17&gt;0,C17/H17,""))</f>
+        <v/>
+      </c>
+      <c r="K17" s="24" t="str">
+        <f aca="false">IF(A17="","",G17*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L17" s="11"/>
+      <c r="M17" s="12" t="str">
+        <f aca="false">IF(A17="","",(G17+H17)*30*L17)</f>
+        <v/>
+      </c>
+      <c r="N17" s="6" t="str">
+        <f aca="false">IF(A17="","",IF(OR(AND(G17&gt;0,B17&lt;=0),AND(H17&gt;0,C17&lt;=0)),"RUPTURA",IF(OR(AND(G17&gt;0,B17&lt;=K17),AND(H17&gt;0,C17&lt;=H17*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G17+H17=0,"Sem giro: revisar",IF(OR(AND(G17&gt;0,I17&gt;120),AND(H17&gt;0,J17&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O17" s="25"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16"/>
-      <c r="B18" s="16"/>
+      <c r="B18" s="14"/>
       <c r="C18" s="14"/>
       <c r="D18" s="14"/>
-      <c r="E18" s="18" t="str">
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="18" t="str">
+        <f aca="false">IF(A18="","",(E18+F18)/30)</f>
+        <v/>
+      </c>
+      <c r="H18" s="18" t="str">
         <f aca="false">IF(A18="","",D18/30)</f>
         <v/>
       </c>
-      <c r="F18" s="24" t="str">
-        <f aca="false">IF(A18="","",IF(E18&gt;0,C18/E18,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G18" s="24" t="str">
-        <f aca="false">IF(A18="","",E18*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H18" s="11"/>
-      <c r="I18" s="12" t="str">
-        <f aca="false">IF(A18="","",E18*30*H18)</f>
-        <v/>
-      </c>
-      <c r="J18" s="6" t="str">
-        <f aca="false">IF(A18="","",IF(C18&lt;=0,"RUPTURA",IF(F18="sem giro","Sem giro: revisar",IF(C18&lt;=G18,"REPOR (abaixo do ponto)",IF(F18&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K18" s="25"/>
+      <c r="I18" s="24" t="str">
+        <f aca="false">IF(A18="","",IF(G18&gt;0,B18/G18,""))</f>
+        <v/>
+      </c>
+      <c r="J18" s="24" t="str">
+        <f aca="false">IF(A18="","",IF(H18&gt;0,C18/H18,""))</f>
+        <v/>
+      </c>
+      <c r="K18" s="24" t="str">
+        <f aca="false">IF(A18="","",G18*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L18" s="11"/>
+      <c r="M18" s="12" t="str">
+        <f aca="false">IF(A18="","",(G18+H18)*30*L18)</f>
+        <v/>
+      </c>
+      <c r="N18" s="6" t="str">
+        <f aca="false">IF(A18="","",IF(OR(AND(G18&gt;0,B18&lt;=0),AND(H18&gt;0,C18&lt;=0)),"RUPTURA",IF(OR(AND(G18&gt;0,B18&lt;=K18),AND(H18&gt;0,C18&lt;=H18*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G18+H18=0,"Sem giro: revisar",IF(OR(AND(G18&gt;0,I18&gt;120),AND(H18&gt;0,J18&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O18" s="25"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="16"/>
-      <c r="B19" s="16"/>
+      <c r="B19" s="14"/>
       <c r="C19" s="14"/>
       <c r="D19" s="14"/>
-      <c r="E19" s="18" t="str">
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="18" t="str">
+        <f aca="false">IF(A19="","",(E19+F19)/30)</f>
+        <v/>
+      </c>
+      <c r="H19" s="18" t="str">
         <f aca="false">IF(A19="","",D19/30)</f>
         <v/>
       </c>
-      <c r="F19" s="24" t="str">
-        <f aca="false">IF(A19="","",IF(E19&gt;0,C19/E19,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G19" s="24" t="str">
-        <f aca="false">IF(A19="","",E19*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H19" s="11"/>
-      <c r="I19" s="12" t="str">
-        <f aca="false">IF(A19="","",E19*30*H19)</f>
-        <v/>
-      </c>
-      <c r="J19" s="6" t="str">
-        <f aca="false">IF(A19="","",IF(C19&lt;=0,"RUPTURA",IF(F19="sem giro","Sem giro: revisar",IF(C19&lt;=G19,"REPOR (abaixo do ponto)",IF(F19&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K19" s="25"/>
+      <c r="I19" s="24" t="str">
+        <f aca="false">IF(A19="","",IF(G19&gt;0,B19/G19,""))</f>
+        <v/>
+      </c>
+      <c r="J19" s="24" t="str">
+        <f aca="false">IF(A19="","",IF(H19&gt;0,C19/H19,""))</f>
+        <v/>
+      </c>
+      <c r="K19" s="24" t="str">
+        <f aca="false">IF(A19="","",G19*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L19" s="11"/>
+      <c r="M19" s="12" t="str">
+        <f aca="false">IF(A19="","",(G19+H19)*30*L19)</f>
+        <v/>
+      </c>
+      <c r="N19" s="6" t="str">
+        <f aca="false">IF(A19="","",IF(OR(AND(G19&gt;0,B19&lt;=0),AND(H19&gt;0,C19&lt;=0)),"RUPTURA",IF(OR(AND(G19&gt;0,B19&lt;=K19),AND(H19&gt;0,C19&lt;=H19*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G19+H19=0,"Sem giro: revisar",IF(OR(AND(G19&gt;0,I19&gt;120),AND(H19&gt;0,J19&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O19" s="25"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16"/>
-      <c r="B20" s="16"/>
+      <c r="B20" s="14"/>
       <c r="C20" s="14"/>
       <c r="D20" s="14"/>
-      <c r="E20" s="18" t="str">
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="18" t="str">
+        <f aca="false">IF(A20="","",(E20+F20)/30)</f>
+        <v/>
+      </c>
+      <c r="H20" s="18" t="str">
         <f aca="false">IF(A20="","",D20/30)</f>
         <v/>
       </c>
-      <c r="F20" s="24" t="str">
-        <f aca="false">IF(A20="","",IF(E20&gt;0,C20/E20,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G20" s="24" t="str">
-        <f aca="false">IF(A20="","",E20*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H20" s="11"/>
-      <c r="I20" s="12" t="str">
-        <f aca="false">IF(A20="","",E20*30*H20)</f>
-        <v/>
-      </c>
-      <c r="J20" s="6" t="str">
-        <f aca="false">IF(A20="","",IF(C20&lt;=0,"RUPTURA",IF(F20="sem giro","Sem giro: revisar",IF(C20&lt;=G20,"REPOR (abaixo do ponto)",IF(F20&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K20" s="25"/>
+      <c r="I20" s="24" t="str">
+        <f aca="false">IF(A20="","",IF(G20&gt;0,B20/G20,""))</f>
+        <v/>
+      </c>
+      <c r="J20" s="24" t="str">
+        <f aca="false">IF(A20="","",IF(H20&gt;0,C20/H20,""))</f>
+        <v/>
+      </c>
+      <c r="K20" s="24" t="str">
+        <f aca="false">IF(A20="","",G20*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L20" s="11"/>
+      <c r="M20" s="12" t="str">
+        <f aca="false">IF(A20="","",(G20+H20)*30*L20)</f>
+        <v/>
+      </c>
+      <c r="N20" s="6" t="str">
+        <f aca="false">IF(A20="","",IF(OR(AND(G20&gt;0,B20&lt;=0),AND(H20&gt;0,C20&lt;=0)),"RUPTURA",IF(OR(AND(G20&gt;0,B20&lt;=K20),AND(H20&gt;0,C20&lt;=H20*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G20+H20=0,"Sem giro: revisar",IF(OR(AND(G20&gt;0,I20&gt;120),AND(H20&gt;0,J20&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O20" s="25"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16"/>
-      <c r="B21" s="16"/>
+      <c r="B21" s="14"/>
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
-      <c r="E21" s="18" t="str">
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="18" t="str">
+        <f aca="false">IF(A21="","",(E21+F21)/30)</f>
+        <v/>
+      </c>
+      <c r="H21" s="18" t="str">
         <f aca="false">IF(A21="","",D21/30)</f>
         <v/>
       </c>
-      <c r="F21" s="24" t="str">
-        <f aca="false">IF(A21="","",IF(E21&gt;0,C21/E21,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G21" s="24" t="str">
-        <f aca="false">IF(A21="","",E21*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H21" s="11"/>
-      <c r="I21" s="12" t="str">
-        <f aca="false">IF(A21="","",E21*30*H21)</f>
-        <v/>
-      </c>
-      <c r="J21" s="6" t="str">
-        <f aca="false">IF(A21="","",IF(C21&lt;=0,"RUPTURA",IF(F21="sem giro","Sem giro: revisar",IF(C21&lt;=G21,"REPOR (abaixo do ponto)",IF(F21&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K21" s="25"/>
+      <c r="I21" s="24" t="str">
+        <f aca="false">IF(A21="","",IF(G21&gt;0,B21/G21,""))</f>
+        <v/>
+      </c>
+      <c r="J21" s="24" t="str">
+        <f aca="false">IF(A21="","",IF(H21&gt;0,C21/H21,""))</f>
+        <v/>
+      </c>
+      <c r="K21" s="24" t="str">
+        <f aca="false">IF(A21="","",G21*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L21" s="11"/>
+      <c r="M21" s="12" t="str">
+        <f aca="false">IF(A21="","",(G21+H21)*30*L21)</f>
+        <v/>
+      </c>
+      <c r="N21" s="6" t="str">
+        <f aca="false">IF(A21="","",IF(OR(AND(G21&gt;0,B21&lt;=0),AND(H21&gt;0,C21&lt;=0)),"RUPTURA",IF(OR(AND(G21&gt;0,B21&lt;=K21),AND(H21&gt;0,C21&lt;=H21*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G21+H21=0,"Sem giro: revisar",IF(OR(AND(G21&gt;0,I21&gt;120),AND(H21&gt;0,J21&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O21" s="25"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16"/>
-      <c r="B22" s="16"/>
+      <c r="B22" s="14"/>
       <c r="C22" s="14"/>
       <c r="D22" s="14"/>
-      <c r="E22" s="18" t="str">
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="18" t="str">
+        <f aca="false">IF(A22="","",(E22+F22)/30)</f>
+        <v/>
+      </c>
+      <c r="H22" s="18" t="str">
         <f aca="false">IF(A22="","",D22/30)</f>
         <v/>
       </c>
-      <c r="F22" s="24" t="str">
-        <f aca="false">IF(A22="","",IF(E22&gt;0,C22/E22,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G22" s="24" t="str">
-        <f aca="false">IF(A22="","",E22*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H22" s="11"/>
-      <c r="I22" s="12" t="str">
-        <f aca="false">IF(A22="","",E22*30*H22)</f>
-        <v/>
-      </c>
-      <c r="J22" s="6" t="str">
-        <f aca="false">IF(A22="","",IF(C22&lt;=0,"RUPTURA",IF(F22="sem giro","Sem giro: revisar",IF(C22&lt;=G22,"REPOR (abaixo do ponto)",IF(F22&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K22" s="25"/>
+      <c r="I22" s="24" t="str">
+        <f aca="false">IF(A22="","",IF(G22&gt;0,B22/G22,""))</f>
+        <v/>
+      </c>
+      <c r="J22" s="24" t="str">
+        <f aca="false">IF(A22="","",IF(H22&gt;0,C22/H22,""))</f>
+        <v/>
+      </c>
+      <c r="K22" s="24" t="str">
+        <f aca="false">IF(A22="","",G22*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L22" s="11"/>
+      <c r="M22" s="12" t="str">
+        <f aca="false">IF(A22="","",(G22+H22)*30*L22)</f>
+        <v/>
+      </c>
+      <c r="N22" s="6" t="str">
+        <f aca="false">IF(A22="","",IF(OR(AND(G22&gt;0,B22&lt;=0),AND(H22&gt;0,C22&lt;=0)),"RUPTURA",IF(OR(AND(G22&gt;0,B22&lt;=K22),AND(H22&gt;0,C22&lt;=H22*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G22+H22=0,"Sem giro: revisar",IF(OR(AND(G22&gt;0,I22&gt;120),AND(H22&gt;0,J22&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O22" s="25"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="16"/>
-      <c r="B23" s="16"/>
+      <c r="B23" s="14"/>
       <c r="C23" s="14"/>
       <c r="D23" s="14"/>
-      <c r="E23" s="18" t="str">
+      <c r="E23" s="14"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="18" t="str">
+        <f aca="false">IF(A23="","",(E23+F23)/30)</f>
+        <v/>
+      </c>
+      <c r="H23" s="18" t="str">
         <f aca="false">IF(A23="","",D23/30)</f>
         <v/>
       </c>
-      <c r="F23" s="24" t="str">
-        <f aca="false">IF(A23="","",IF(E23&gt;0,C23/E23,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G23" s="24" t="str">
-        <f aca="false">IF(A23="","",E23*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H23" s="11"/>
-      <c r="I23" s="12" t="str">
-        <f aca="false">IF(A23="","",E23*30*H23)</f>
-        <v/>
-      </c>
-      <c r="J23" s="6" t="str">
-        <f aca="false">IF(A23="","",IF(C23&lt;=0,"RUPTURA",IF(F23="sem giro","Sem giro: revisar",IF(C23&lt;=G23,"REPOR (abaixo do ponto)",IF(F23&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K23" s="25"/>
+      <c r="I23" s="24" t="str">
+        <f aca="false">IF(A23="","",IF(G23&gt;0,B23/G23,""))</f>
+        <v/>
+      </c>
+      <c r="J23" s="24" t="str">
+        <f aca="false">IF(A23="","",IF(H23&gt;0,C23/H23,""))</f>
+        <v/>
+      </c>
+      <c r="K23" s="24" t="str">
+        <f aca="false">IF(A23="","",G23*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L23" s="11"/>
+      <c r="M23" s="12" t="str">
+        <f aca="false">IF(A23="","",(G23+H23)*30*L23)</f>
+        <v/>
+      </c>
+      <c r="N23" s="6" t="str">
+        <f aca="false">IF(A23="","",IF(OR(AND(G23&gt;0,B23&lt;=0),AND(H23&gt;0,C23&lt;=0)),"RUPTURA",IF(OR(AND(G23&gt;0,B23&lt;=K23),AND(H23&gt;0,C23&lt;=H23*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G23+H23=0,"Sem giro: revisar",IF(OR(AND(G23&gt;0,I23&gt;120),AND(H23&gt;0,J23&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O23" s="25"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="16"/>
-      <c r="B24" s="16"/>
+      <c r="B24" s="14"/>
       <c r="C24" s="14"/>
       <c r="D24" s="14"/>
-      <c r="E24" s="18" t="str">
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="18" t="str">
+        <f aca="false">IF(A24="","",(E24+F24)/30)</f>
+        <v/>
+      </c>
+      <c r="H24" s="18" t="str">
         <f aca="false">IF(A24="","",D24/30)</f>
         <v/>
       </c>
-      <c r="F24" s="24" t="str">
-        <f aca="false">IF(A24="","",IF(E24&gt;0,C24/E24,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G24" s="24" t="str">
-        <f aca="false">IF(A24="","",E24*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H24" s="11"/>
-      <c r="I24" s="12" t="str">
-        <f aca="false">IF(A24="","",E24*30*H24)</f>
-        <v/>
-      </c>
-      <c r="J24" s="6" t="str">
-        <f aca="false">IF(A24="","",IF(C24&lt;=0,"RUPTURA",IF(F24="sem giro","Sem giro: revisar",IF(C24&lt;=G24,"REPOR (abaixo do ponto)",IF(F24&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K24" s="25"/>
+      <c r="I24" s="24" t="str">
+        <f aca="false">IF(A24="","",IF(G24&gt;0,B24/G24,""))</f>
+        <v/>
+      </c>
+      <c r="J24" s="24" t="str">
+        <f aca="false">IF(A24="","",IF(H24&gt;0,C24/H24,""))</f>
+        <v/>
+      </c>
+      <c r="K24" s="24" t="str">
+        <f aca="false">IF(A24="","",G24*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L24" s="11"/>
+      <c r="M24" s="12" t="str">
+        <f aca="false">IF(A24="","",(G24+H24)*30*L24)</f>
+        <v/>
+      </c>
+      <c r="N24" s="6" t="str">
+        <f aca="false">IF(A24="","",IF(OR(AND(G24&gt;0,B24&lt;=0),AND(H24&gt;0,C24&lt;=0)),"RUPTURA",IF(OR(AND(G24&gt;0,B24&lt;=K24),AND(H24&gt;0,C24&lt;=H24*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G24+H24=0,"Sem giro: revisar",IF(OR(AND(G24&gt;0,I24&gt;120),AND(H24&gt;0,J24&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O24" s="25"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16"/>
-      <c r="B25" s="16"/>
+      <c r="B25" s="14"/>
       <c r="C25" s="14"/>
       <c r="D25" s="14"/>
-      <c r="E25" s="18" t="str">
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="18" t="str">
+        <f aca="false">IF(A25="","",(E25+F25)/30)</f>
+        <v/>
+      </c>
+      <c r="H25" s="18" t="str">
         <f aca="false">IF(A25="","",D25/30)</f>
         <v/>
       </c>
-      <c r="F25" s="24" t="str">
-        <f aca="false">IF(A25="","",IF(E25&gt;0,C25/E25,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G25" s="24" t="str">
-        <f aca="false">IF(A25="","",E25*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H25" s="11"/>
-      <c r="I25" s="12" t="str">
-        <f aca="false">IF(A25="","",E25*30*H25)</f>
-        <v/>
-      </c>
-      <c r="J25" s="6" t="str">
-        <f aca="false">IF(A25="","",IF(C25&lt;=0,"RUPTURA",IF(F25="sem giro","Sem giro: revisar",IF(C25&lt;=G25,"REPOR (abaixo do ponto)",IF(F25&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K25" s="25"/>
+      <c r="I25" s="24" t="str">
+        <f aca="false">IF(A25="","",IF(G25&gt;0,B25/G25,""))</f>
+        <v/>
+      </c>
+      <c r="J25" s="24" t="str">
+        <f aca="false">IF(A25="","",IF(H25&gt;0,C25/H25,""))</f>
+        <v/>
+      </c>
+      <c r="K25" s="24" t="str">
+        <f aca="false">IF(A25="","",G25*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L25" s="11"/>
+      <c r="M25" s="12" t="str">
+        <f aca="false">IF(A25="","",(G25+H25)*30*L25)</f>
+        <v/>
+      </c>
+      <c r="N25" s="6" t="str">
+        <f aca="false">IF(A25="","",IF(OR(AND(G25&gt;0,B25&lt;=0),AND(H25&gt;0,C25&lt;=0)),"RUPTURA",IF(OR(AND(G25&gt;0,B25&lt;=K25),AND(H25&gt;0,C25&lt;=H25*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G25+H25=0,"Sem giro: revisar",IF(OR(AND(G25&gt;0,I25&gt;120),AND(H25&gt;0,J25&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O25" s="25"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16"/>
-      <c r="B26" s="16"/>
+      <c r="B26" s="14"/>
       <c r="C26" s="14"/>
       <c r="D26" s="14"/>
-      <c r="E26" s="18" t="str">
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="18" t="str">
+        <f aca="false">IF(A26="","",(E26+F26)/30)</f>
+        <v/>
+      </c>
+      <c r="H26" s="18" t="str">
         <f aca="false">IF(A26="","",D26/30)</f>
         <v/>
       </c>
-      <c r="F26" s="24" t="str">
-        <f aca="false">IF(A26="","",IF(E26&gt;0,C26/E26,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G26" s="24" t="str">
-        <f aca="false">IF(A26="","",E26*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H26" s="11"/>
-      <c r="I26" s="12" t="str">
-        <f aca="false">IF(A26="","",E26*30*H26)</f>
-        <v/>
-      </c>
-      <c r="J26" s="6" t="str">
-        <f aca="false">IF(A26="","",IF(C26&lt;=0,"RUPTURA",IF(F26="sem giro","Sem giro: revisar",IF(C26&lt;=G26,"REPOR (abaixo do ponto)",IF(F26&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K26" s="25"/>
+      <c r="I26" s="24" t="str">
+        <f aca="false">IF(A26="","",IF(G26&gt;0,B26/G26,""))</f>
+        <v/>
+      </c>
+      <c r="J26" s="24" t="str">
+        <f aca="false">IF(A26="","",IF(H26&gt;0,C26/H26,""))</f>
+        <v/>
+      </c>
+      <c r="K26" s="24" t="str">
+        <f aca="false">IF(A26="","",G26*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L26" s="11"/>
+      <c r="M26" s="12" t="str">
+        <f aca="false">IF(A26="","",(G26+H26)*30*L26)</f>
+        <v/>
+      </c>
+      <c r="N26" s="6" t="str">
+        <f aca="false">IF(A26="","",IF(OR(AND(G26&gt;0,B26&lt;=0),AND(H26&gt;0,C26&lt;=0)),"RUPTURA",IF(OR(AND(G26&gt;0,B26&lt;=K26),AND(H26&gt;0,C26&lt;=H26*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G26+H26=0,"Sem giro: revisar",IF(OR(AND(G26&gt;0,I26&gt;120),AND(H26&gt;0,J26&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O26" s="25"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="16"/>
-      <c r="B27" s="16"/>
+      <c r="B27" s="14"/>
       <c r="C27" s="14"/>
       <c r="D27" s="14"/>
-      <c r="E27" s="18" t="str">
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="18" t="str">
+        <f aca="false">IF(A27="","",(E27+F27)/30)</f>
+        <v/>
+      </c>
+      <c r="H27" s="18" t="str">
         <f aca="false">IF(A27="","",D27/30)</f>
         <v/>
       </c>
-      <c r="F27" s="24" t="str">
-        <f aca="false">IF(A27="","",IF(E27&gt;0,C27/E27,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G27" s="24" t="str">
-        <f aca="false">IF(A27="","",E27*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H27" s="11"/>
-      <c r="I27" s="12" t="str">
-        <f aca="false">IF(A27="","",E27*30*H27)</f>
-        <v/>
-      </c>
-      <c r="J27" s="6" t="str">
-        <f aca="false">IF(A27="","",IF(C27&lt;=0,"RUPTURA",IF(F27="sem giro","Sem giro: revisar",IF(C27&lt;=G27,"REPOR (abaixo do ponto)",IF(F27&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K27" s="25"/>
+      <c r="I27" s="24" t="str">
+        <f aca="false">IF(A27="","",IF(G27&gt;0,B27/G27,""))</f>
+        <v/>
+      </c>
+      <c r="J27" s="24" t="str">
+        <f aca="false">IF(A27="","",IF(H27&gt;0,C27/H27,""))</f>
+        <v/>
+      </c>
+      <c r="K27" s="24" t="str">
+        <f aca="false">IF(A27="","",G27*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L27" s="11"/>
+      <c r="M27" s="12" t="str">
+        <f aca="false">IF(A27="","",(G27+H27)*30*L27)</f>
+        <v/>
+      </c>
+      <c r="N27" s="6" t="str">
+        <f aca="false">IF(A27="","",IF(OR(AND(G27&gt;0,B27&lt;=0),AND(H27&gt;0,C27&lt;=0)),"RUPTURA",IF(OR(AND(G27&gt;0,B27&lt;=K27),AND(H27&gt;0,C27&lt;=H27*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G27+H27=0,"Sem giro: revisar",IF(OR(AND(G27&gt;0,I27&gt;120),AND(H27&gt;0,J27&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O27" s="25"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16"/>
-      <c r="B28" s="16"/>
+      <c r="B28" s="14"/>
       <c r="C28" s="14"/>
       <c r="D28" s="14"/>
-      <c r="E28" s="18" t="str">
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="18" t="str">
+        <f aca="false">IF(A28="","",(E28+F28)/30)</f>
+        <v/>
+      </c>
+      <c r="H28" s="18" t="str">
         <f aca="false">IF(A28="","",D28/30)</f>
         <v/>
       </c>
-      <c r="F28" s="24" t="str">
-        <f aca="false">IF(A28="","",IF(E28&gt;0,C28/E28,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G28" s="24" t="str">
-        <f aca="false">IF(A28="","",E28*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H28" s="11"/>
-      <c r="I28" s="12" t="str">
-        <f aca="false">IF(A28="","",E28*30*H28)</f>
-        <v/>
-      </c>
-      <c r="J28" s="6" t="str">
-        <f aca="false">IF(A28="","",IF(C28&lt;=0,"RUPTURA",IF(F28="sem giro","Sem giro: revisar",IF(C28&lt;=G28,"REPOR (abaixo do ponto)",IF(F28&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K28" s="25"/>
+      <c r="I28" s="24" t="str">
+        <f aca="false">IF(A28="","",IF(G28&gt;0,B28/G28,""))</f>
+        <v/>
+      </c>
+      <c r="J28" s="24" t="str">
+        <f aca="false">IF(A28="","",IF(H28&gt;0,C28/H28,""))</f>
+        <v/>
+      </c>
+      <c r="K28" s="24" t="str">
+        <f aca="false">IF(A28="","",G28*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L28" s="11"/>
+      <c r="M28" s="12" t="str">
+        <f aca="false">IF(A28="","",(G28+H28)*30*L28)</f>
+        <v/>
+      </c>
+      <c r="N28" s="6" t="str">
+        <f aca="false">IF(A28="","",IF(OR(AND(G28&gt;0,B28&lt;=0),AND(H28&gt;0,C28&lt;=0)),"RUPTURA",IF(OR(AND(G28&gt;0,B28&lt;=K28),AND(H28&gt;0,C28&lt;=H28*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G28+H28=0,"Sem giro: revisar",IF(OR(AND(G28&gt;0,I28&gt;120),AND(H28&gt;0,J28&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O28" s="25"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16"/>
-      <c r="B29" s="16"/>
+      <c r="B29" s="14"/>
       <c r="C29" s="14"/>
       <c r="D29" s="14"/>
-      <c r="E29" s="18" t="str">
+      <c r="E29" s="14"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="18" t="str">
+        <f aca="false">IF(A29="","",(E29+F29)/30)</f>
+        <v/>
+      </c>
+      <c r="H29" s="18" t="str">
         <f aca="false">IF(A29="","",D29/30)</f>
         <v/>
       </c>
-      <c r="F29" s="24" t="str">
-        <f aca="false">IF(A29="","",IF(E29&gt;0,C29/E29,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G29" s="24" t="str">
-        <f aca="false">IF(A29="","",E29*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H29" s="11"/>
-      <c r="I29" s="12" t="str">
-        <f aca="false">IF(A29="","",E29*30*H29)</f>
-        <v/>
-      </c>
-      <c r="J29" s="6" t="str">
-        <f aca="false">IF(A29="","",IF(C29&lt;=0,"RUPTURA",IF(F29="sem giro","Sem giro: revisar",IF(C29&lt;=G29,"REPOR (abaixo do ponto)",IF(F29&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K29" s="25"/>
+      <c r="I29" s="24" t="str">
+        <f aca="false">IF(A29="","",IF(G29&gt;0,B29/G29,""))</f>
+        <v/>
+      </c>
+      <c r="J29" s="24" t="str">
+        <f aca="false">IF(A29="","",IF(H29&gt;0,C29/H29,""))</f>
+        <v/>
+      </c>
+      <c r="K29" s="24" t="str">
+        <f aca="false">IF(A29="","",G29*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L29" s="11"/>
+      <c r="M29" s="12" t="str">
+        <f aca="false">IF(A29="","",(G29+H29)*30*L29)</f>
+        <v/>
+      </c>
+      <c r="N29" s="6" t="str">
+        <f aca="false">IF(A29="","",IF(OR(AND(G29&gt;0,B29&lt;=0),AND(H29&gt;0,C29&lt;=0)),"RUPTURA",IF(OR(AND(G29&gt;0,B29&lt;=K29),AND(H29&gt;0,C29&lt;=H29*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G29+H29=0,"Sem giro: revisar",IF(OR(AND(G29&gt;0,I29&gt;120),AND(H29&gt;0,J29&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O29" s="25"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16"/>
-      <c r="B30" s="16"/>
+      <c r="B30" s="14"/>
       <c r="C30" s="14"/>
       <c r="D30" s="14"/>
-      <c r="E30" s="18" t="str">
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="18" t="str">
+        <f aca="false">IF(A30="","",(E30+F30)/30)</f>
+        <v/>
+      </c>
+      <c r="H30" s="18" t="str">
         <f aca="false">IF(A30="","",D30/30)</f>
         <v/>
       </c>
-      <c r="F30" s="24" t="str">
-        <f aca="false">IF(A30="","",IF(E30&gt;0,C30/E30,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G30" s="24" t="str">
-        <f aca="false">IF(A30="","",E30*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H30" s="11"/>
-      <c r="I30" s="12" t="str">
-        <f aca="false">IF(A30="","",E30*30*H30)</f>
-        <v/>
-      </c>
-      <c r="J30" s="6" t="str">
-        <f aca="false">IF(A30="","",IF(C30&lt;=0,"RUPTURA",IF(F30="sem giro","Sem giro: revisar",IF(C30&lt;=G30,"REPOR (abaixo do ponto)",IF(F30&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K30" s="25"/>
+      <c r="I30" s="24" t="str">
+        <f aca="false">IF(A30="","",IF(G30&gt;0,B30/G30,""))</f>
+        <v/>
+      </c>
+      <c r="J30" s="24" t="str">
+        <f aca="false">IF(A30="","",IF(H30&gt;0,C30/H30,""))</f>
+        <v/>
+      </c>
+      <c r="K30" s="24" t="str">
+        <f aca="false">IF(A30="","",G30*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L30" s="11"/>
+      <c r="M30" s="12" t="str">
+        <f aca="false">IF(A30="","",(G30+H30)*30*L30)</f>
+        <v/>
+      </c>
+      <c r="N30" s="6" t="str">
+        <f aca="false">IF(A30="","",IF(OR(AND(G30&gt;0,B30&lt;=0),AND(H30&gt;0,C30&lt;=0)),"RUPTURA",IF(OR(AND(G30&gt;0,B30&lt;=K30),AND(H30&gt;0,C30&lt;=H30*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G30+H30=0,"Sem giro: revisar",IF(OR(AND(G30&gt;0,I30&gt;120),AND(H30&gt;0,J30&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O30" s="25"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="16"/>
-      <c r="B31" s="16"/>
+      <c r="B31" s="14"/>
       <c r="C31" s="14"/>
       <c r="D31" s="14"/>
-      <c r="E31" s="18" t="str">
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="18" t="str">
+        <f aca="false">IF(A31="","",(E31+F31)/30)</f>
+        <v/>
+      </c>
+      <c r="H31" s="18" t="str">
         <f aca="false">IF(A31="","",D31/30)</f>
         <v/>
       </c>
-      <c r="F31" s="24" t="str">
-        <f aca="false">IF(A31="","",IF(E31&gt;0,C31/E31,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G31" s="24" t="str">
-        <f aca="false">IF(A31="","",E31*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H31" s="11"/>
-      <c r="I31" s="12" t="str">
-        <f aca="false">IF(A31="","",E31*30*H31)</f>
-        <v/>
-      </c>
-      <c r="J31" s="6" t="str">
-        <f aca="false">IF(A31="","",IF(C31&lt;=0,"RUPTURA",IF(F31="sem giro","Sem giro: revisar",IF(C31&lt;=G31,"REPOR (abaixo do ponto)",IF(F31&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K31" s="25"/>
+      <c r="I31" s="24" t="str">
+        <f aca="false">IF(A31="","",IF(G31&gt;0,B31/G31,""))</f>
+        <v/>
+      </c>
+      <c r="J31" s="24" t="str">
+        <f aca="false">IF(A31="","",IF(H31&gt;0,C31/H31,""))</f>
+        <v/>
+      </c>
+      <c r="K31" s="24" t="str">
+        <f aca="false">IF(A31="","",G31*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L31" s="11"/>
+      <c r="M31" s="12" t="str">
+        <f aca="false">IF(A31="","",(G31+H31)*30*L31)</f>
+        <v/>
+      </c>
+      <c r="N31" s="6" t="str">
+        <f aca="false">IF(A31="","",IF(OR(AND(G31&gt;0,B31&lt;=0),AND(H31&gt;0,C31&lt;=0)),"RUPTURA",IF(OR(AND(G31&gt;0,B31&lt;=K31),AND(H31&gt;0,C31&lt;=H31*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G31+H31=0,"Sem giro: revisar",IF(OR(AND(G31&gt;0,I31&gt;120),AND(H31&gt;0,J31&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O31" s="25"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16"/>
-      <c r="B32" s="16"/>
+      <c r="B32" s="14"/>
       <c r="C32" s="14"/>
       <c r="D32" s="14"/>
-      <c r="E32" s="18" t="str">
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="18" t="str">
+        <f aca="false">IF(A32="","",(E32+F32)/30)</f>
+        <v/>
+      </c>
+      <c r="H32" s="18" t="str">
         <f aca="false">IF(A32="","",D32/30)</f>
         <v/>
       </c>
-      <c r="F32" s="24" t="str">
-        <f aca="false">IF(A32="","",IF(E32&gt;0,C32/E32,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G32" s="24" t="str">
-        <f aca="false">IF(A32="","",E32*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H32" s="11"/>
-      <c r="I32" s="12" t="str">
-        <f aca="false">IF(A32="","",E32*30*H32)</f>
-        <v/>
-      </c>
-      <c r="J32" s="6" t="str">
-        <f aca="false">IF(A32="","",IF(C32&lt;=0,"RUPTURA",IF(F32="sem giro","Sem giro: revisar",IF(C32&lt;=G32,"REPOR (abaixo do ponto)",IF(F32&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K32" s="25"/>
+      <c r="I32" s="24" t="str">
+        <f aca="false">IF(A32="","",IF(G32&gt;0,B32/G32,""))</f>
+        <v/>
+      </c>
+      <c r="J32" s="24" t="str">
+        <f aca="false">IF(A32="","",IF(H32&gt;0,C32/H32,""))</f>
+        <v/>
+      </c>
+      <c r="K32" s="24" t="str">
+        <f aca="false">IF(A32="","",G32*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L32" s="11"/>
+      <c r="M32" s="12" t="str">
+        <f aca="false">IF(A32="","",(G32+H32)*30*L32)</f>
+        <v/>
+      </c>
+      <c r="N32" s="6" t="str">
+        <f aca="false">IF(A32="","",IF(OR(AND(G32&gt;0,B32&lt;=0),AND(H32&gt;0,C32&lt;=0)),"RUPTURA",IF(OR(AND(G32&gt;0,B32&lt;=K32),AND(H32&gt;0,C32&lt;=H32*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G32+H32=0,"Sem giro: revisar",IF(OR(AND(G32&gt;0,I32&gt;120),AND(H32&gt;0,J32&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O32" s="25"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16"/>
-      <c r="B33" s="16"/>
+      <c r="B33" s="14"/>
       <c r="C33" s="14"/>
       <c r="D33" s="14"/>
-      <c r="E33" s="18" t="str">
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="18" t="str">
+        <f aca="false">IF(A33="","",(E33+F33)/30)</f>
+        <v/>
+      </c>
+      <c r="H33" s="18" t="str">
         <f aca="false">IF(A33="","",D33/30)</f>
         <v/>
       </c>
-      <c r="F33" s="24" t="str">
-        <f aca="false">IF(A33="","",IF(E33&gt;0,C33/E33,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G33" s="24" t="str">
-        <f aca="false">IF(A33="","",E33*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H33" s="11"/>
-      <c r="I33" s="12" t="str">
-        <f aca="false">IF(A33="","",E33*30*H33)</f>
-        <v/>
-      </c>
-      <c r="J33" s="6" t="str">
-        <f aca="false">IF(A33="","",IF(C33&lt;=0,"RUPTURA",IF(F33="sem giro","Sem giro: revisar",IF(C33&lt;=G33,"REPOR (abaixo do ponto)",IF(F33&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K33" s="25"/>
+      <c r="I33" s="24" t="str">
+        <f aca="false">IF(A33="","",IF(G33&gt;0,B33/G33,""))</f>
+        <v/>
+      </c>
+      <c r="J33" s="24" t="str">
+        <f aca="false">IF(A33="","",IF(H33&gt;0,C33/H33,""))</f>
+        <v/>
+      </c>
+      <c r="K33" s="24" t="str">
+        <f aca="false">IF(A33="","",G33*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L33" s="11"/>
+      <c r="M33" s="12" t="str">
+        <f aca="false">IF(A33="","",(G33+H33)*30*L33)</f>
+        <v/>
+      </c>
+      <c r="N33" s="6" t="str">
+        <f aca="false">IF(A33="","",IF(OR(AND(G33&gt;0,B33&lt;=0),AND(H33&gt;0,C33&lt;=0)),"RUPTURA",IF(OR(AND(G33&gt;0,B33&lt;=K33),AND(H33&gt;0,C33&lt;=H33*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G33+H33=0,"Sem giro: revisar",IF(OR(AND(G33&gt;0,I33&gt;120),AND(H33&gt;0,J33&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O33" s="25"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="16"/>
-      <c r="B34" s="16"/>
+      <c r="B34" s="14"/>
       <c r="C34" s="14"/>
       <c r="D34" s="14"/>
-      <c r="E34" s="18" t="str">
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="18" t="str">
+        <f aca="false">IF(A34="","",(E34+F34)/30)</f>
+        <v/>
+      </c>
+      <c r="H34" s="18" t="str">
         <f aca="false">IF(A34="","",D34/30)</f>
         <v/>
       </c>
-      <c r="F34" s="24" t="str">
-        <f aca="false">IF(A34="","",IF(E34&gt;0,C34/E34,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G34" s="24" t="str">
-        <f aca="false">IF(A34="","",E34*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H34" s="11"/>
-      <c r="I34" s="12" t="str">
-        <f aca="false">IF(A34="","",E34*30*H34)</f>
-        <v/>
-      </c>
-      <c r="J34" s="6" t="str">
-        <f aca="false">IF(A34="","",IF(C34&lt;=0,"RUPTURA",IF(F34="sem giro","Sem giro: revisar",IF(C34&lt;=G34,"REPOR (abaixo do ponto)",IF(F34&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K34" s="25"/>
+      <c r="I34" s="24" t="str">
+        <f aca="false">IF(A34="","",IF(G34&gt;0,B34/G34,""))</f>
+        <v/>
+      </c>
+      <c r="J34" s="24" t="str">
+        <f aca="false">IF(A34="","",IF(H34&gt;0,C34/H34,""))</f>
+        <v/>
+      </c>
+      <c r="K34" s="24" t="str">
+        <f aca="false">IF(A34="","",G34*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L34" s="11"/>
+      <c r="M34" s="12" t="str">
+        <f aca="false">IF(A34="","",(G34+H34)*30*L34)</f>
+        <v/>
+      </c>
+      <c r="N34" s="6" t="str">
+        <f aca="false">IF(A34="","",IF(OR(AND(G34&gt;0,B34&lt;=0),AND(H34&gt;0,C34&lt;=0)),"RUPTURA",IF(OR(AND(G34&gt;0,B34&lt;=K34),AND(H34&gt;0,C34&lt;=H34*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G34+H34=0,"Sem giro: revisar",IF(OR(AND(G34&gt;0,I34&gt;120),AND(H34&gt;0,J34&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O34" s="25"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16"/>
-      <c r="B35" s="16"/>
+      <c r="B35" s="14"/>
       <c r="C35" s="14"/>
       <c r="D35" s="14"/>
-      <c r="E35" s="18" t="str">
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="18" t="str">
+        <f aca="false">IF(A35="","",(E35+F35)/30)</f>
+        <v/>
+      </c>
+      <c r="H35" s="18" t="str">
         <f aca="false">IF(A35="","",D35/30)</f>
         <v/>
       </c>
-      <c r="F35" s="24" t="str">
-        <f aca="false">IF(A35="","",IF(E35&gt;0,C35/E35,"sem giro"))</f>
-        <v/>
-      </c>
-      <c r="G35" s="24" t="str">
-        <f aca="false">IF(A35="","",E35*(Parametros!$B$17+Parametros!$B$19))</f>
-        <v/>
-      </c>
-      <c r="H35" s="11"/>
-      <c r="I35" s="12" t="str">
-        <f aca="false">IF(A35="","",E35*30*H35)</f>
-        <v/>
-      </c>
-      <c r="J35" s="6" t="str">
-        <f aca="false">IF(A35="","",IF(C35&lt;=0,"RUPTURA",IF(F35="sem giro","Sem giro: revisar",IF(C35&lt;=G35,"REPOR (abaixo do ponto)",IF(F35&gt;120,"Excesso (&gt;120 dias)","OK")))))</f>
-        <v/>
-      </c>
-      <c r="K35" s="25"/>
+      <c r="I35" s="24" t="str">
+        <f aca="false">IF(A35="","",IF(G35&gt;0,B35/G35,""))</f>
+        <v/>
+      </c>
+      <c r="J35" s="24" t="str">
+        <f aca="false">IF(A35="","",IF(H35&gt;0,C35/H35,""))</f>
+        <v/>
+      </c>
+      <c r="K35" s="24" t="str">
+        <f aca="false">IF(A35="","",G35*(Parametros!$B$17+Parametros!$B$19))</f>
+        <v/>
+      </c>
+      <c r="L35" s="11"/>
+      <c r="M35" s="12" t="str">
+        <f aca="false">IF(A35="","",(G35+H35)*30*L35)</f>
+        <v/>
+      </c>
+      <c r="N35" s="6" t="str">
+        <f aca="false">IF(A35="","",IF(OR(AND(G35&gt;0,B35&lt;=0),AND(H35&gt;0,C35&lt;=0)),"RUPTURA",IF(OR(AND(G35&gt;0,B35&lt;=K35),AND(H35&gt;0,C35&lt;=H35*(Parametros!$B$17+Parametros!$B$19))),"REPOR (abaixo do ponto)",IF(G35+H35=0,"Sem giro: revisar",IF(OR(AND(G35&gt;0,I35&gt;120),AND(H35&gt;0,J35&gt;120)),"Excesso (&gt;120 dias)","OK")))))</f>
+        <v/>
+      </c>
+      <c r="O35" s="25"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="26" t="s">
-        <v>121</v>
-      </c>
-      <c r="I37" s="21" t="n">
-        <f aca="false">SUM(I6:I35)</f>
-        <v>1200</v>
+        <v>127</v>
+      </c>
+      <c r="M37" s="21" t="n">
+        <f aca="false">SUM(M6:M35)</f>
+        <v>1600</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="I38" s="12" t="n">
+        <v>128</v>
+      </c>
+      <c r="M38" s="12" t="n">
         <f aca="false">Parametros!$B$16+Parametros!$B$21</f>
         <v>500</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="I39" s="21" t="n">
-        <f aca="false">I38-I37</f>
-        <v>-700</v>
+        <v>129</v>
+      </c>
+      <c r="M39" s="21" t="n">
+        <f aca="false">M38-M37</f>
+        <v>-1100</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="J6:J35">
+  <conditionalFormatting sqref="N6:N35">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>OR(J6="RUPTURA",LEFT(J6,5)="REPOR")</formula>
+      <formula>OR(N6="RUPTURA",LEFT(N6,5)="REPOR")</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"OK"</formula>
@@ -5648,17 +6038,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B3" s="11" t="n">
         <v>0</v>
@@ -5666,24 +6056,24 @@
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -5692,7 +6082,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="12" t="n">
@@ -5710,7 +6100,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
@@ -5719,7 +6109,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">Parametros!$B$11</f>
@@ -5740,7 +6130,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
@@ -5749,7 +6139,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B10" s="21" t="n">
         <f aca="false">B5-SUM(B6:B9)</f>
@@ -5770,7 +6160,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B11" s="21" t="n">
         <f aca="false">$B$3+B10</f>
@@ -5791,7 +6181,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
@@ -5800,7 +6190,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">B12</f>
@@ -5821,7 +6211,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">MAX(0,Parametros!$B$21-B13)</f>
@@ -5842,12 +6232,12 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -5871,7 +6261,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -5880,34 +6270,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B5" s="14"/>
       <c r="C5" s="14"/>
@@ -5919,7 +6309,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
@@ -5931,7 +6321,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
@@ -5943,7 +6333,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
@@ -5955,7 +6345,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
@@ -5967,7 +6357,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
@@ -5979,7 +6369,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
@@ -5991,7 +6381,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">B6*Parametros!$B$4</f>
@@ -6012,7 +6402,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
@@ -6024,7 +6414,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B14" s="21" t="n">
         <f aca="false">B6-SUM(B7:B13)</f>
@@ -6045,7 +6435,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B15" s="17" t="str">
         <f aca="false">IF(B6&gt;0,B14/B6,"")</f>
@@ -6066,7 +6456,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B16" s="12" t="n">
         <f aca="false">Parametros!$B$11</f>
@@ -6087,7 +6477,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B17" s="21" t="n">
         <f aca="false">B14-B16</f>
@@ -6108,7 +6498,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">SUM($B17:B17)</f>
@@ -6129,7 +6519,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">Parametros!$B$7-B18</f>
@@ -6150,7 +6540,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B20" s="17" t="n">
         <f aca="false">IF(Parametros!$B$7&gt;0,B18/Parametros!$B$7,"")</f>
@@ -6171,7 +6561,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B21" s="12" t="str">
         <f aca="false">IF(B5&gt;0,B6/B5,"")</f>
@@ -6192,7 +6582,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B22" s="17" t="str">
         <f aca="false">IF(B6&gt;0,B13/B6,"")</f>
@@ -6213,7 +6603,57 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>164</v>
+        <v>170</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="26" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="12" t="n">
+        <f aca="false">SUM(B27:D27)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="12" t="n">
+        <f aca="false">SUM(B28:D28)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B29" s="12" t="n">
+        <f aca="false">B6-B27-B28</f>
+        <v>0</v>
+      </c>
+      <c r="C29" s="12" t="n">
+        <f aca="false">C6-C27-C28</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="12" t="n">
+        <f aca="false">D6-D27-D28</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="12" t="n">
+        <f aca="false">E6-E27-E28</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -6249,17 +6689,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="28" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="B4" s="12" t="n">
         <f aca="false">Parametros!$B$7/Parametros!$B$8</f>
@@ -6268,7 +6708,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="B5" s="12" t="n">
         <f aca="false">Parametros!$B$11</f>
@@ -6277,7 +6717,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="28" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="B6" s="21" t="n">
         <f aca="false">B4+B5</f>
@@ -6286,7 +6726,7 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="29" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="B7" s="12" t="n">
         <f aca="false">2*Parametros!$B$7/(Parametros!$B$8+1)</f>
@@ -6295,7 +6735,7 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="29" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="B8" s="21" t="n">
         <f aca="false">B7+B5</f>
@@ -6304,25 +6744,25 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6414,7 +6854,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>